<commit_message>
Add structural alignment evaluation script for Design2Code-18B-V0. Implement DOM adaptation, scoring metrics, and results reporting in Excel format. Update README with new metrics and summary statistics. Include debug screenshots for evaluation cases.
</commit_message>
<xml_diff>
--- a/design2code-18b-v0/evaluation_results/iou_scores.xlsx
+++ b/design2code-18b-v0/evaluation_results/iou_scores.xlsx
@@ -447,7 +447,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.08445751687679294</v>
+        <v>0.05134755444786486</v>
       </c>
     </row>
     <row r="3">
@@ -457,7 +457,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1050222674637437</v>
+        <v>0.1014903897643338</v>
       </c>
     </row>
     <row r="4">
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.05700731075250506</v>
+        <v>0.04674590514765344</v>
       </c>
     </row>
     <row r="5">
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.07051912697581601</v>
+        <v>0.06968615415455512</v>
       </c>
     </row>
     <row r="6">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.0683793473012328</v>
+        <v>0.1024301991291484</v>
       </c>
     </row>
     <row r="7">
@@ -497,7 +497,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.05804429390498882</v>
+        <v>0.03989048530678253</v>
       </c>
     </row>
     <row r="8">
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.02453791213022608</v>
+        <v>0.02319126266457221</v>
       </c>
     </row>
     <row r="9">
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.06697570018647458</v>
+        <v>0.07140766377714482</v>
       </c>
     </row>
     <row r="10">
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.005159653491958975</v>
+        <v>0.00358778480567726</v>
       </c>
     </row>
     <row r="11">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.04179360642710957</v>
+        <v>0.0261665672062389</v>
       </c>
     </row>
     <row r="12">
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.01621563414068904</v>
+        <v>0.01620734167652354</v>
       </c>
     </row>
     <row r="13">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1885729336400064</v>
+        <v>0.1796640291774187</v>
       </c>
     </row>
     <row r="14">
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.01831072840498627</v>
+        <v>0.02043242658813808</v>
       </c>
     </row>
     <row r="16">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.03073306479770232</v>
+        <v>0.04396106864263459</v>
       </c>
     </row>
     <row r="17">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.09288823546532034</v>
+        <v>0.0829898708523799</v>
       </c>
     </row>
     <row r="19">
@@ -617,7 +617,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.05642681741224435</v>
+        <v>0.07597697694436852</v>
       </c>
     </row>
     <row r="20">
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.04806553412130129</v>
+        <v>0.05142092703225967</v>
       </c>
     </row>
     <row r="21">
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.02245891963364229</v>
+        <v>0.03786582545329591</v>
       </c>
     </row>
     <row r="22">
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.1101730969360644</v>
+        <v>0.101170661784897</v>
       </c>
     </row>
     <row r="23">
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.05798412346096327</v>
+        <v>0.07101726986760931</v>
       </c>
     </row>
     <row r="24">
@@ -677,7 +677,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.1578626922471388</v>
+        <v>0.111494405096134</v>
       </c>
     </row>
     <row r="26">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.08398481862431172</v>
+        <v>0.09164505162350194</v>
       </c>
     </row>
     <row r="27">
@@ -697,7 +697,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.004884470830585483</v>
+        <v>0.006551186464030947</v>
       </c>
     </row>
     <row r="28">
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.01311516021571692</v>
+        <v>0.0128677380322735</v>
       </c>
     </row>
     <row r="29">
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.0260291307721768</v>
+        <v>0.02691094067499085</v>
       </c>
     </row>
     <row r="30">
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.1172921929110884</v>
+        <v>0.07589092132146001</v>
       </c>
     </row>
     <row r="31">
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.05976898581316448</v>
+        <v>0.05038301466842739</v>
       </c>
     </row>
     <row r="32">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.01137828303015354</v>
+        <v>0.01263001720743036</v>
       </c>
     </row>
     <row r="33">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0.05472997483945721</v>
+        <v>0.05986420688992944</v>
       </c>
     </row>
     <row r="34">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.01939976559023541</v>
+        <v>0.0244275354443925</v>
       </c>
     </row>
     <row r="35">
@@ -777,7 +777,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.005949550297682473</v>
+        <v>0.01833584596208234</v>
       </c>
     </row>
     <row r="36">
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.04166165139522139</v>
+        <v>0.02782230638329327</v>
       </c>
     </row>
     <row r="37">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.1312872918359093</v>
+        <v>0.2360276610810076</v>
       </c>
     </row>
     <row r="38">
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.1167895366960293</v>
+        <v>0.1074123602167478</v>
       </c>
     </row>
     <row r="39">
@@ -817,7 +817,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.04815399938227489</v>
+        <v>0.04354998874612579</v>
       </c>
     </row>
     <row r="40">
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.006818363149720657</v>
+        <v>0.007661221799391069</v>
       </c>
     </row>
     <row r="41">
@@ -837,7 +837,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.1190525384002148</v>
+        <v>0.1227554565921946</v>
       </c>
     </row>
     <row r="42">
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.008855586071951615</v>
+        <v>0.1095461288194616</v>
       </c>
     </row>
     <row r="43">
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.01734501151407918</v>
+        <v>0.07609670903245533</v>
       </c>
     </row>
     <row r="44">
@@ -867,7 +867,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.05831203533979838</v>
+        <v>0.1180059091711297</v>
       </c>
     </row>
     <row r="45">
@@ -877,7 +877,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.08533045668445567</v>
+        <v>0.1242790717772571</v>
       </c>
     </row>
     <row r="46">
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.01073652221392521</v>
+        <v>0.01759410569624674</v>
       </c>
     </row>
     <row r="47">
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.0203577903610683</v>
+        <v>0.02247801664321289</v>
       </c>
     </row>
     <row r="48">
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.02445629727965021</v>
+        <v>0.02383726393173214</v>
       </c>
     </row>
     <row r="49">
@@ -917,7 +917,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0.01625808536829603</v>
+        <v>0.01615784618446613</v>
       </c>
     </row>
     <row r="50">
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0.03296326674466747</v>
+        <v>0.006770057605290907</v>
       </c>
     </row>
     <row r="51">
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0.056761258765416</v>
+        <v>0.05552660545954176</v>
       </c>
     </row>
     <row r="52">
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0.0199570984227304</v>
+        <v>0.02314746135542888</v>
       </c>
     </row>
     <row r="53">
@@ -957,7 +957,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.04745765548218448</v>
+        <v>0.0460986752735657</v>
       </c>
     </row>
     <row r="54">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>0.05321701067340784</v>
+        <v>0.06999956736664419</v>
       </c>
     </row>
     <row r="55">
@@ -977,7 +977,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0.06472649238464384</v>
+        <v>0.06183401845617189</v>
       </c>
     </row>
     <row r="56">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.003848616981040418</v>
+        <v>0.005114075352960082</v>
       </c>
     </row>
     <row r="57">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>0.06233211590205776</v>
+        <v>0.07271078136469866</v>
       </c>
     </row>
     <row r="58">
@@ -1017,7 +1017,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>0.03056860064083449</v>
+        <v>0.02730175511195892</v>
       </c>
     </row>
     <row r="60">
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.03366914094798542</v>
+        <v>0.03230332704781318</v>
       </c>
     </row>
     <row r="61">
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>0.01442359198013653</v>
+        <v>0.01158219824001276</v>
       </c>
     </row>
     <row r="62">
@@ -1047,7 +1047,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>0.06993989293230381</v>
+        <v>0.06651010408592944</v>
       </c>
     </row>
     <row r="63">
@@ -1057,7 +1057,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>0.0592610136857256</v>
+        <v>0.06316767479480628</v>
       </c>
     </row>
     <row r="64">
@@ -1067,7 +1067,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>0.0608093509256292</v>
+        <v>0.05925013679933102</v>
       </c>
     </row>
     <row r="65">
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.03721920574345855</v>
+        <v>0.03039128874020515</v>
       </c>
     </row>
     <row r="66">
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>0.2561218532128997</v>
+        <v>0.06213455891740074</v>
       </c>
     </row>
     <row r="67">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>0.006690770024343331</v>
+        <v>0.03547782519733163</v>
       </c>
     </row>
     <row r="68">
@@ -1117,7 +1117,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>0</v>
+        <v>0.01422302934761605</v>
       </c>
     </row>
     <row r="70">
@@ -1127,7 +1127,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>0.05362144641419606</v>
+        <v>0.0521319617915795</v>
       </c>
     </row>
     <row r="71">
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0.00421783959038992</v>
+        <v>0.003120045724398023</v>
       </c>
     </row>
     <row r="72">
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>0.07038616585343799</v>
+        <v>0.06040099052875397</v>
       </c>
     </row>
     <row r="73">
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>0.06210428994555155</v>
+        <v>0.07273213790251642</v>
       </c>
     </row>
     <row r="74">
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>0.1191930035977268</v>
+        <v>0.1592629973842256</v>
       </c>
     </row>
     <row r="75">
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>0.03535227873415775</v>
+        <v>0.03912791663633923</v>
       </c>
     </row>
     <row r="76">
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>0.2225428731700479</v>
+        <v>0.2836089368663589</v>
       </c>
     </row>
     <row r="77">
@@ -1197,7 +1197,7 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>0.03735165989867256</v>
+        <v>0.02628458504708931</v>
       </c>
     </row>
     <row r="78">
@@ -1207,7 +1207,7 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>0.04908449710986147</v>
+        <v>0.05867721416740881</v>
       </c>
     </row>
     <row r="79">
@@ -1217,7 +1217,7 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>0.09991634479423188</v>
+        <v>0.1138570390388535</v>
       </c>
     </row>
     <row r="80">
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>0.04609725922675623</v>
+        <v>0.03280206956873437</v>
       </c>
     </row>
     <row r="81">
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>0.06680532866725183</v>
+        <v>0.06692387196920591</v>
       </c>
     </row>
     <row r="82">
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>0.13624167085401</v>
+        <v>0.1611011254409812</v>
       </c>
     </row>
     <row r="83">
@@ -1257,7 +1257,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0.02207780238486998</v>
+        <v>0.02002505586033505</v>
       </c>
     </row>
     <row r="84">
@@ -1267,7 +1267,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0.07533658327465877</v>
+        <v>0.06219306383560161</v>
       </c>
     </row>
     <row r="85">
@@ -1277,7 +1277,7 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>0.01542179492400262</v>
+        <v>0.03391633620377789</v>
       </c>
     </row>
     <row r="86">
@@ -1287,7 +1287,7 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0.1713446284068213</v>
+        <v>0.1641822887326032</v>
       </c>
     </row>
     <row r="87">
@@ -1297,7 +1297,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0.04377162108472644</v>
+        <v>0.03984465070838782</v>
       </c>
     </row>
     <row r="88">
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>0.02158201456716647</v>
+        <v>0.01679716858469103</v>
       </c>
     </row>
     <row r="89">
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>0.01504495095794811</v>
+        <v>0.01470861350574691</v>
       </c>
     </row>
     <row r="90">
@@ -1327,7 +1327,7 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>0.1348850722024041</v>
+        <v>0.1403766086278063</v>
       </c>
     </row>
     <row r="91">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>0.07193218393160762</v>
+        <v>0.0579573685751102</v>
       </c>
     </row>
     <row r="92">
@@ -1347,7 +1347,7 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>0.01506873274125125</v>
+        <v>0.01494364728414133</v>
       </c>
     </row>
     <row r="93">
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>0.04214124684853069</v>
+        <v>0.04261759458638211</v>
       </c>
     </row>
     <row r="94">
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>0.07593396034340794</v>
+        <v>0.07773356445574225</v>
       </c>
     </row>
     <row r="95">
@@ -1377,7 +1377,7 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>0.06835274134365131</v>
+        <v>0.08173030902532925</v>
       </c>
     </row>
     <row r="96">
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>0.02114920434405303</v>
+        <v>0.01915101375656999</v>
       </c>
     </row>
     <row r="97">
@@ -1397,7 +1397,7 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>0.04951040048045003</v>
+        <v>0.05197872701274756</v>
       </c>
     </row>
     <row r="98">
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>0.008994948311891656</v>
+        <v>0.01144462086183384</v>
       </c>
     </row>
     <row r="99">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>0.07859989214995959</v>
+        <v>0.0773118363165028</v>
       </c>
     </row>
     <row r="100">
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>0.08618919627802904</v>
+        <v>0.0651714152359478</v>
       </c>
     </row>
     <row r="101">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>0.02180041090746252</v>
+        <v>0.07606329312440326</v>
       </c>
     </row>
     <row r="102">
@@ -1447,7 +1447,7 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>0.006193970924535108</v>
+        <v>0.002874903804186898</v>
       </c>
     </row>
     <row r="103">
@@ -1457,7 +1457,7 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>0.06669725162938434</v>
+        <v>0.07746812404201299</v>
       </c>
     </row>
     <row r="104">
@@ -1467,7 +1467,7 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>0.05059698207269447</v>
+        <v>0.02306644109730581</v>
       </c>
     </row>
     <row r="105">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>0.009110264603826029</v>
+        <v>0.01277780606931123</v>
       </c>
     </row>
     <row r="107">
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>0.0439199360365949</v>
+        <v>0.05564235268433307</v>
       </c>
     </row>
     <row r="108">
@@ -1507,7 +1507,7 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>0.02795106226904593</v>
+        <v>0.03701749369035906</v>
       </c>
     </row>
     <row r="109">
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>0.1002140360817192</v>
+        <v>0.08669382958594068</v>
       </c>
     </row>
     <row r="110">
@@ -1527,7 +1527,7 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>0.01803198487772131</v>
+        <v>0.02356741518494351</v>
       </c>
     </row>
     <row r="111">
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>0.03330503874811562</v>
+        <v>0.05881267475253225</v>
       </c>
     </row>
     <row r="112">
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>0.01886074398672832</v>
+        <v>0.01937681892961064</v>
       </c>
     </row>
     <row r="113">
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>0.08972339007990596</v>
+        <v>0.1040373421760337</v>
       </c>
     </row>
     <row r="114">
@@ -1567,7 +1567,7 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>0.00723083022316723</v>
+        <v>0.01160252211501756</v>
       </c>
     </row>
     <row r="115">
@@ -1577,7 +1577,7 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>0.05081052401072385</v>
+        <v>0.04749609488784992</v>
       </c>
     </row>
     <row r="116">
@@ -1587,7 +1587,7 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>0.01172672819903688</v>
+        <v>0.0119352124644408</v>
       </c>
     </row>
     <row r="117">
@@ -1597,7 +1597,7 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>0.04867955049910023</v>
+        <v>0.04286438374910398</v>
       </c>
     </row>
     <row r="118">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>0.04142248427223968</v>
+        <v>0.05709698392735892</v>
       </c>
     </row>
     <row r="119">
@@ -1617,7 +1617,7 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>0.04464925852289326</v>
+        <v>0.02533831433060985</v>
       </c>
     </row>
     <row r="120">
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>0.05233737162575554</v>
+        <v>0.05334281544870161</v>
       </c>
     </row>
     <row r="121">
@@ -1637,7 +1637,7 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>0.006953634880348078</v>
+        <v>0.003068535390808119</v>
       </c>
     </row>
     <row r="122">
@@ -1647,7 +1647,7 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>0.02519173990759935</v>
+        <v>0.1055653955159132</v>
       </c>
     </row>
     <row r="123">
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="B123" t="n">
-        <v>0.01528131072802121</v>
+        <v>0.01402495491831719</v>
       </c>
     </row>
     <row r="124">
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="B124" t="n">
-        <v>0.05833726123398909</v>
+        <v>0.08115695792166029</v>
       </c>
     </row>
     <row r="125">
@@ -1677,7 +1677,7 @@
         </is>
       </c>
       <c r="B125" t="n">
-        <v>0.07835382574517384</v>
+        <v>0.05153872424014368</v>
       </c>
     </row>
     <row r="126">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="B126" t="n">
-        <v>0.024121535493701</v>
+        <v>0.0266948674104868</v>
       </c>
     </row>
     <row r="127">
@@ -1697,7 +1697,7 @@
         </is>
       </c>
       <c r="B127" t="n">
-        <v>0.0222734924105527</v>
+        <v>0.01759421713668659</v>
       </c>
     </row>
     <row r="128">
@@ -1707,7 +1707,7 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>0.05155708290460411</v>
+        <v>0.05904398860737576</v>
       </c>
     </row>
     <row r="129">
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="B129" t="n">
-        <v>0.004464654584463618</v>
+        <v>0.009009760102419606</v>
       </c>
     </row>
     <row r="130">
@@ -1727,7 +1727,7 @@
         </is>
       </c>
       <c r="B130" t="n">
-        <v>0.04943191168254753</v>
+        <v>0.064940325686778</v>
       </c>
     </row>
     <row r="131">
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="B131" t="n">
-        <v>0.04094770573029567</v>
+        <v>0.193362517029628</v>
       </c>
     </row>
     <row r="132">
@@ -1747,7 +1747,7 @@
         </is>
       </c>
       <c r="B132" t="n">
-        <v>0.07186689027884788</v>
+        <v>0.05829357035538173</v>
       </c>
     </row>
     <row r="133">
@@ -1767,7 +1767,7 @@
         </is>
       </c>
       <c r="B134" t="n">
-        <v>0.0214367159854684</v>
+        <v>0.01631363033615486</v>
       </c>
     </row>
     <row r="135">
@@ -1777,7 +1777,7 @@
         </is>
       </c>
       <c r="B135" t="n">
-        <v>0.0002534309044513005</v>
+        <v>0.001515461424993706</v>
       </c>
     </row>
     <row r="136">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="B136" t="n">
-        <v>0.04164708427996787</v>
+        <v>0.04282571331246435</v>
       </c>
     </row>
     <row r="137">
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>0.005469904991602623</v>
+        <v>0.005509093200907326</v>
       </c>
     </row>
     <row r="138">
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="B138" t="n">
-        <v>0.01718188433832467</v>
+        <v>0.01950404745071456</v>
       </c>
     </row>
     <row r="139">
@@ -1817,7 +1817,7 @@
         </is>
       </c>
       <c r="B139" t="n">
-        <v>0.004154283265772727</v>
+        <v>0.00527856754191606</v>
       </c>
     </row>
     <row r="140">
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="B140" t="n">
-        <v>0.04114481677388498</v>
+        <v>0.04246568807000727</v>
       </c>
     </row>
     <row r="141">
@@ -1837,7 +1837,7 @@
         </is>
       </c>
       <c r="B141" t="n">
-        <v>0.03997024660998715</v>
+        <v>0.05056742356168581</v>
       </c>
     </row>
     <row r="142">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="B142" t="n">
-        <v>0.02525584115127047</v>
+        <v>0.03920223562065663</v>
       </c>
     </row>
     <row r="143">
@@ -1857,7 +1857,7 @@
         </is>
       </c>
       <c r="B143" t="n">
-        <v>0.02318972616304915</v>
+        <v>0.02436009630091038</v>
       </c>
     </row>
     <row r="144">
@@ -1867,7 +1867,7 @@
         </is>
       </c>
       <c r="B144" t="n">
-        <v>0.00877527590305247</v>
+        <v>0.002140304838763128</v>
       </c>
     </row>
     <row r="145">
@@ -1877,7 +1877,7 @@
         </is>
       </c>
       <c r="B145" t="n">
-        <v>0.06221247938888586</v>
+        <v>0.04871529731043408</v>
       </c>
     </row>
     <row r="146">
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="B146" t="n">
-        <v>0.03410128769009137</v>
+        <v>0.02923530729557648</v>
       </c>
     </row>
     <row r="147">
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="B147" t="n">
-        <v>0.08000171018308676</v>
+        <v>0.07966276035567001</v>
       </c>
     </row>
     <row r="148">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="B148" t="n">
-        <v>0.01270267097253612</v>
+        <v>0.01254373252347789</v>
       </c>
     </row>
     <row r="149">
@@ -1917,7 +1917,7 @@
         </is>
       </c>
       <c r="B149" t="n">
-        <v>0.005273636826709664</v>
+        <v>0.005206736090263518</v>
       </c>
     </row>
     <row r="150">
@@ -1927,7 +1927,7 @@
         </is>
       </c>
       <c r="B150" t="n">
-        <v>0.0446391892160378</v>
+        <v>0.04899765562457404</v>
       </c>
     </row>
     <row r="151">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="B151" t="n">
-        <v>0.03578735449393992</v>
+        <v>0.04190999997143956</v>
       </c>
     </row>
     <row r="152">
@@ -1947,7 +1947,7 @@
         </is>
       </c>
       <c r="B152" t="n">
-        <v>0.1377153893362923</v>
+        <v>0.1365830098518232</v>
       </c>
     </row>
     <row r="153">
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="B153" t="n">
-        <v>0.02464647545463852</v>
+        <v>0.01851769155365434</v>
       </c>
     </row>
     <row r="154">
@@ -1967,7 +1967,7 @@
         </is>
       </c>
       <c r="B154" t="n">
-        <v>0.04524899535974558</v>
+        <v>0.04887513750650058</v>
       </c>
     </row>
     <row r="155">
@@ -1977,7 +1977,7 @@
         </is>
       </c>
       <c r="B155" t="n">
-        <v>0.01757568955755445</v>
+        <v>0.01064429775082058</v>
       </c>
     </row>
     <row r="156">
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="B156" t="n">
-        <v>0.06567683410818641</v>
+        <v>0.04273658551000159</v>
       </c>
     </row>
     <row r="157">
@@ -1997,7 +1997,7 @@
         </is>
       </c>
       <c r="B157" t="n">
-        <v>0.0818931146417857</v>
+        <v>0.09081534743376399</v>
       </c>
     </row>
     <row r="158">
@@ -2007,7 +2007,7 @@
         </is>
       </c>
       <c r="B158" t="n">
-        <v>0.003408828139205464</v>
+        <v>0.01321265134044672</v>
       </c>
     </row>
     <row r="159">
@@ -2017,7 +2017,7 @@
         </is>
       </c>
       <c r="B159" t="n">
-        <v>0.04709238639399679</v>
+        <v>0.03826023828273568</v>
       </c>
     </row>
     <row r="160">
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="B160" t="n">
-        <v>0.06142825345825478</v>
+        <v>0.06617763929013189</v>
       </c>
     </row>
     <row r="161">
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="B161" t="n">
-        <v>0.05719642041534941</v>
+        <v>0.0506635854947652</v>
       </c>
     </row>
     <row r="162">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="B162" t="n">
-        <v>0.04730589836087019</v>
+        <v>0.04812852239575097</v>
       </c>
     </row>
     <row r="163">
@@ -2057,7 +2057,7 @@
         </is>
       </c>
       <c r="B163" t="n">
-        <v>0.03862160758045225</v>
+        <v>0.03909630874271292</v>
       </c>
     </row>
     <row r="164">
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="B164" t="n">
-        <v>0.01741272222370676</v>
+        <v>0.03319418895261873</v>
       </c>
     </row>
     <row r="165">
@@ -2077,7 +2077,7 @@
         </is>
       </c>
       <c r="B165" t="n">
-        <v>0.05879340200491935</v>
+        <v>0.04407485556323599</v>
       </c>
     </row>
     <row r="166">
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="B166" t="n">
-        <v>0.0321681564826045</v>
+        <v>0.03327985389059664</v>
       </c>
     </row>
     <row r="167">
@@ -2097,7 +2097,7 @@
         </is>
       </c>
       <c r="B167" t="n">
-        <v>0.04628133678294296</v>
+        <v>0.08202239906555132</v>
       </c>
     </row>
     <row r="168">
@@ -2107,7 +2107,7 @@
         </is>
       </c>
       <c r="B168" t="n">
-        <v>0.04614457926683176</v>
+        <v>0.06513315619484453</v>
       </c>
     </row>
     <row r="169">
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="B169" t="n">
-        <v>0.02701194290415735</v>
+        <v>0.02594000156084749</v>
       </c>
     </row>
     <row r="170">
@@ -2127,7 +2127,7 @@
         </is>
       </c>
       <c r="B170" t="n">
-        <v>0</v>
+        <v>0.000127097674983443</v>
       </c>
     </row>
     <row r="171">
@@ -2137,7 +2137,7 @@
         </is>
       </c>
       <c r="B171" t="n">
-        <v>0.01657653756068498</v>
+        <v>0.02929478372420099</v>
       </c>
     </row>
     <row r="172">
@@ -2147,7 +2147,7 @@
         </is>
       </c>
       <c r="B172" t="n">
-        <v>0.03175363071609205</v>
+        <v>0.03297754521894145</v>
       </c>
     </row>
     <row r="173">
@@ -2157,7 +2157,7 @@
         </is>
       </c>
       <c r="B173" t="n">
-        <v>0.0380967202701389</v>
+        <v>0.04324794548517514</v>
       </c>
     </row>
     <row r="174">
@@ -2167,7 +2167,7 @@
         </is>
       </c>
       <c r="B174" t="n">
-        <v>0.07813241518709049</v>
+        <v>0.09261996291704036</v>
       </c>
     </row>
     <row r="175">
@@ -2187,7 +2187,7 @@
         </is>
       </c>
       <c r="B176" t="n">
-        <v>0.02755833645550806</v>
+        <v>0.01776999811830111</v>
       </c>
     </row>
     <row r="177">
@@ -2197,7 +2197,7 @@
         </is>
       </c>
       <c r="B177" t="n">
-        <v>0.004337563836221419</v>
+        <v>0.008080916005068281</v>
       </c>
     </row>
     <row r="178">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="B178" t="n">
-        <v>0.02787456445993031</v>
+        <v>0.02772429726607624</v>
       </c>
     </row>
     <row r="179">
@@ -2227,7 +2227,7 @@
         </is>
       </c>
       <c r="B180" t="n">
-        <v>0.04942698616016756</v>
+        <v>0.05023237538109274</v>
       </c>
     </row>
     <row r="181">
@@ -2237,7 +2237,7 @@
         </is>
       </c>
       <c r="B181" t="n">
-        <v>0.09056417930535964</v>
+        <v>0.1266013186850364</v>
       </c>
     </row>
     <row r="182">
@@ -2247,7 +2247,7 @@
         </is>
       </c>
       <c r="B182" t="n">
-        <v>0.08869359950728009</v>
+        <v>0.1014393864394245</v>
       </c>
     </row>
     <row r="183">
@@ -2257,7 +2257,7 @@
         </is>
       </c>
       <c r="B183" t="n">
-        <v>0.1369562514816646</v>
+        <v>0.148428346473611</v>
       </c>
     </row>
     <row r="184">
@@ -2267,7 +2267,7 @@
         </is>
       </c>
       <c r="B184" t="n">
-        <v>0.06976577654049684</v>
+        <v>0.08612670327591757</v>
       </c>
     </row>
     <row r="185">
@@ -2277,7 +2277,7 @@
         </is>
       </c>
       <c r="B185" t="n">
-        <v>0.01907078346697417</v>
+        <v>0.02094173175487246</v>
       </c>
     </row>
     <row r="186">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="B186" t="n">
-        <v>0.004617838952734375</v>
+        <v>0.002101852624900667</v>
       </c>
     </row>
     <row r="187">
@@ -2297,7 +2297,7 @@
         </is>
       </c>
       <c r="B187" t="n">
-        <v>0</v>
+        <v>0.001730606490250652</v>
       </c>
     </row>
     <row r="188">
@@ -2307,7 +2307,7 @@
         </is>
       </c>
       <c r="B188" t="n">
-        <v>0.2171215069992355</v>
+        <v>0.2395509556592278</v>
       </c>
     </row>
     <row r="189">
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="B189" t="n">
-        <v>0.08819122664043333</v>
+        <v>0.08433607596627511</v>
       </c>
     </row>
     <row r="190">
@@ -2327,7 +2327,7 @@
         </is>
       </c>
       <c r="B190" t="n">
-        <v>0.02618055068218558</v>
+        <v>0.02872786939817806</v>
       </c>
     </row>
     <row r="191">
@@ -2337,7 +2337,7 @@
         </is>
       </c>
       <c r="B191" t="n">
-        <v>0.01136027320374725</v>
+        <v>0.005749402309907535</v>
       </c>
     </row>
     <row r="192">
@@ -2347,7 +2347,7 @@
         </is>
       </c>
       <c r="B192" t="n">
-        <v>0.04775994905305782</v>
+        <v>0.03885758476669594</v>
       </c>
     </row>
     <row r="193">
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="B193" t="n">
-        <v>0.08821633905939259</v>
+        <v>0.08313544992123775</v>
       </c>
     </row>
     <row r="194">
@@ -2367,7 +2367,7 @@
         </is>
       </c>
       <c r="B194" t="n">
-        <v>0.01835121217758862</v>
+        <v>0.01286543763916403</v>
       </c>
     </row>
     <row r="195">
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="B195" t="n">
-        <v>0.04139656232722389</v>
+        <v>0.03922753619853601</v>
       </c>
     </row>
     <row r="196">
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="B196" t="n">
-        <v>0.07119781869459078</v>
+        <v>0.04635937575391105</v>
       </c>
     </row>
     <row r="197">
@@ -2397,7 +2397,7 @@
         </is>
       </c>
       <c r="B197" t="n">
-        <v>0.01467082782970075</v>
+        <v>0.01387920768048898</v>
       </c>
     </row>
     <row r="198">
@@ -2407,7 +2407,7 @@
         </is>
       </c>
       <c r="B198" t="n">
-        <v>0.0505051772952494</v>
+        <v>0.04420256709193038</v>
       </c>
     </row>
     <row r="199">
@@ -2417,7 +2417,7 @@
         </is>
       </c>
       <c r="B199" t="n">
-        <v>0.07706558186825471</v>
+        <v>0.02592697097384833</v>
       </c>
     </row>
     <row r="200">
@@ -2427,7 +2427,7 @@
         </is>
       </c>
       <c r="B200" t="n">
-        <v>0.02137534240276722</v>
+        <v>0.02823760589878503</v>
       </c>
     </row>
     <row r="201">
@@ -2437,7 +2437,7 @@
         </is>
       </c>
       <c r="B201" t="n">
-        <v>0.07956015448731431</v>
+        <v>0.05390095215282231</v>
       </c>
     </row>
     <row r="202">
@@ -2447,7 +2447,7 @@
         </is>
       </c>
       <c r="B202" t="n">
-        <v>0.02939461342548441</v>
+        <v>0.01869446959848284</v>
       </c>
     </row>
     <row r="203">
@@ -2457,7 +2457,7 @@
         </is>
       </c>
       <c r="B203" t="n">
-        <v>0.07295528773954393</v>
+        <v>0.07291741117682084</v>
       </c>
     </row>
     <row r="204">
@@ -2467,7 +2467,7 @@
         </is>
       </c>
       <c r="B204" t="n">
-        <v>0.02933581853643314</v>
+        <v>0.02457196349998823</v>
       </c>
     </row>
     <row r="205">
@@ -2477,7 +2477,7 @@
         </is>
       </c>
       <c r="B205" t="n">
-        <v>0.001853367034130401</v>
+        <v>0.001223901835394966</v>
       </c>
     </row>
     <row r="206">
@@ -2487,7 +2487,7 @@
         </is>
       </c>
       <c r="B206" t="n">
-        <v>0.006197994948634117</v>
+        <v>0.02244177977418839</v>
       </c>
     </row>
     <row r="207">
@@ -2507,7 +2507,7 @@
         </is>
       </c>
       <c r="B208" t="n">
-        <v>0.06428533777249815</v>
+        <v>0.05697194731350635</v>
       </c>
     </row>
     <row r="209">
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="B209" t="n">
-        <v>0.02135297932333743</v>
+        <v>0.03339555134815245</v>
       </c>
     </row>
     <row r="210">
@@ -2527,7 +2527,7 @@
         </is>
       </c>
       <c r="B210" t="n">
-        <v>0.04195011750520755</v>
+        <v>0.07490400346564009</v>
       </c>
     </row>
     <row r="211">
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="B211" t="n">
-        <v>0.0461424373116477</v>
+        <v>0.04540657463208835</v>
       </c>
     </row>
     <row r="212">
@@ -2547,7 +2547,7 @@
         </is>
       </c>
       <c r="B212" t="n">
-        <v>0.04896501126202676</v>
+        <v>0.02833030274487904</v>
       </c>
     </row>
     <row r="213">
@@ -2557,7 +2557,7 @@
         </is>
       </c>
       <c r="B213" t="n">
-        <v>0.0027466531703369</v>
+        <v>0.001874753931355164</v>
       </c>
     </row>
     <row r="214">
@@ -2577,7 +2577,7 @@
         </is>
       </c>
       <c r="B215" t="n">
-        <v>0.03476219716432139</v>
+        <v>0.04902956176127102</v>
       </c>
     </row>
     <row r="216">
@@ -2587,7 +2587,7 @@
         </is>
       </c>
       <c r="B216" t="n">
-        <v>0.02644155844632919</v>
+        <v>0.03712235766793482</v>
       </c>
     </row>
     <row r="217">
@@ -2597,7 +2597,7 @@
         </is>
       </c>
       <c r="B217" t="n">
-        <v>0.0272469317344798</v>
+        <v>0.03487312871824241</v>
       </c>
     </row>
     <row r="218">
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="B218" t="n">
-        <v>0.1365478931580106</v>
+        <v>0.10730388541309</v>
       </c>
     </row>
     <row r="219">
@@ -2617,7 +2617,7 @@
         </is>
       </c>
       <c r="B219" t="n">
-        <v>0.0218327673069194</v>
+        <v>0.02327872693452672</v>
       </c>
     </row>
     <row r="220">
@@ -2627,7 +2627,7 @@
         </is>
       </c>
       <c r="B220" t="n">
-        <v>0.04945173673160674</v>
+        <v>0.03305342083806343</v>
       </c>
     </row>
     <row r="221">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="B221" t="n">
-        <v>0.01586212292528789</v>
+        <v>0.01351990399217247</v>
       </c>
     </row>
     <row r="222">
@@ -2647,7 +2647,7 @@
         </is>
       </c>
       <c r="B222" t="n">
-        <v>0.1064024659847133</v>
+        <v>0.1021119056504051</v>
       </c>
     </row>
     <row r="223">
@@ -2657,7 +2657,7 @@
         </is>
       </c>
       <c r="B223" t="n">
-        <v>0.08318417062549809</v>
+        <v>0.09541244164900053</v>
       </c>
     </row>
     <row r="224">
@@ -2667,7 +2667,7 @@
         </is>
       </c>
       <c r="B224" t="n">
-        <v>0.04180167478173232</v>
+        <v>0.04203626556563723</v>
       </c>
     </row>
     <row r="225">
@@ -2677,7 +2677,7 @@
         </is>
       </c>
       <c r="B225" t="n">
-        <v>0.04201193705985887</v>
+        <v>0.04312017116144776</v>
       </c>
     </row>
     <row r="226">
@@ -2687,7 +2687,7 @@
         </is>
       </c>
       <c r="B226" t="n">
-        <v>0.04679008681722077</v>
+        <v>0.04949722449469105</v>
       </c>
     </row>
     <row r="227">
@@ -2697,7 +2697,7 @@
         </is>
       </c>
       <c r="B227" t="n">
-        <v>0.05267808152781332</v>
+        <v>0.0510365652858142</v>
       </c>
     </row>
     <row r="228">
@@ -2707,7 +2707,7 @@
         </is>
       </c>
       <c r="B228" t="n">
-        <v>0.0192842292590592</v>
+        <v>0.01916788769148348</v>
       </c>
     </row>
     <row r="229">
@@ -2717,7 +2717,7 @@
         </is>
       </c>
       <c r="B229" t="n">
-        <v>0.0252668753908221</v>
+        <v>0.02262150612944771</v>
       </c>
     </row>
     <row r="230">
@@ -2727,7 +2727,7 @@
         </is>
       </c>
       <c r="B230" t="n">
-        <v>0.03121484973902771</v>
+        <v>0.03563075157194334</v>
       </c>
     </row>
     <row r="231">
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="B231" t="n">
-        <v>0.04882823663800234</v>
+        <v>0.03512398945120746</v>
       </c>
     </row>
     <row r="232">
@@ -2747,7 +2747,7 @@
         </is>
       </c>
       <c r="B232" t="n">
-        <v>0.08675345217503222</v>
+        <v>0.08903984593906239</v>
       </c>
     </row>
     <row r="233">
@@ -2757,7 +2757,7 @@
         </is>
       </c>
       <c r="B233" t="n">
-        <v>0.003671508125416583</v>
+        <v>0.004255740212859209</v>
       </c>
     </row>
     <row r="234">
@@ -2767,7 +2767,7 @@
         </is>
       </c>
       <c r="B234" t="n">
-        <v>0.02827406335945751</v>
+        <v>0.0609511341076723</v>
       </c>
     </row>
     <row r="235">
@@ -2777,7 +2777,7 @@
         </is>
       </c>
       <c r="B235" t="n">
-        <v>0.0523690322365216</v>
+        <v>0.02480153468881599</v>
       </c>
     </row>
     <row r="236">
@@ -2787,7 +2787,7 @@
         </is>
       </c>
       <c r="B236" t="n">
-        <v>0.05754508294706483</v>
+        <v>0.02502767799229672</v>
       </c>
     </row>
     <row r="237">
@@ -2797,7 +2797,7 @@
         </is>
       </c>
       <c r="B237" t="n">
-        <v>0.1156165562583037</v>
+        <v>0.117374387050641</v>
       </c>
     </row>
     <row r="238">
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="B238" t="n">
-        <v>0.04380647960851178</v>
+        <v>0.08640629938464918</v>
       </c>
     </row>
     <row r="239">
@@ -2817,7 +2817,7 @@
         </is>
       </c>
       <c r="B239" t="n">
-        <v>0.0150884112439919</v>
+        <v>0.03328741834224124</v>
       </c>
     </row>
     <row r="240">
@@ -2827,7 +2827,7 @@
         </is>
       </c>
       <c r="B240" t="n">
-        <v>0.02914146504189723</v>
+        <v>0.02525229205457617</v>
       </c>
     </row>
     <row r="241">
@@ -2837,7 +2837,7 @@
         </is>
       </c>
       <c r="B241" t="n">
-        <v>0.07555484555514026</v>
+        <v>0.06612176807028322</v>
       </c>
     </row>
     <row r="242">
@@ -2847,7 +2847,7 @@
         </is>
       </c>
       <c r="B242" t="n">
-        <v>0.08145222914928145</v>
+        <v>0.05197817238907173</v>
       </c>
     </row>
     <row r="243">
@@ -2857,7 +2857,7 @@
         </is>
       </c>
       <c r="B243" t="n">
-        <v>0.01024798204263657</v>
+        <v>0.008191722625582322</v>
       </c>
     </row>
     <row r="244">
@@ -2867,7 +2867,7 @@
         </is>
       </c>
       <c r="B244" t="n">
-        <v>0.0398972265414087</v>
+        <v>0.02954223361634641</v>
       </c>
     </row>
     <row r="245">
@@ -2877,7 +2877,7 @@
         </is>
       </c>
       <c r="B245" t="n">
-        <v>0.05963081061467958</v>
+        <v>0.06679864755206778</v>
       </c>
     </row>
     <row r="246">
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="B246" t="n">
-        <v>0.06573851035917277</v>
+        <v>0.0708332297582881</v>
       </c>
     </row>
     <row r="247">
@@ -2897,7 +2897,7 @@
         </is>
       </c>
       <c r="B247" t="n">
-        <v>0.04894300486026815</v>
+        <v>0.04661031365601685</v>
       </c>
     </row>
     <row r="248">
@@ -2917,7 +2917,7 @@
         </is>
       </c>
       <c r="B249" t="n">
-        <v>0.07093588683201092</v>
+        <v>0.0605107157129359</v>
       </c>
     </row>
     <row r="250">
@@ -2927,7 +2927,7 @@
         </is>
       </c>
       <c r="B250" t="n">
-        <v>0.149555862172544</v>
+        <v>0.1389352554740336</v>
       </c>
     </row>
     <row r="251">
@@ -2937,7 +2937,7 @@
         </is>
       </c>
       <c r="B251" t="n">
-        <v>0.09540165655392299</v>
+        <v>0.06347676385111696</v>
       </c>
     </row>
     <row r="252">
@@ -2947,7 +2947,7 @@
         </is>
       </c>
       <c r="B252" t="n">
-        <v>0.07771395834573856</v>
+        <v>0.07970736482978004</v>
       </c>
     </row>
     <row r="253">
@@ -2957,7 +2957,7 @@
         </is>
       </c>
       <c r="B253" t="n">
-        <v>0.03898914045386979</v>
+        <v>0.03983388607971956</v>
       </c>
     </row>
     <row r="254">
@@ -2967,7 +2967,7 @@
         </is>
       </c>
       <c r="B254" t="n">
-        <v>0.03018935087538107</v>
+        <v>0.03185363920680049</v>
       </c>
     </row>
     <row r="255">
@@ -2977,7 +2977,7 @@
         </is>
       </c>
       <c r="B255" t="n">
-        <v>0.0126850540261892</v>
+        <v>0.01304958982206243</v>
       </c>
     </row>
     <row r="256">
@@ -2987,7 +2987,7 @@
         </is>
       </c>
       <c r="B256" t="n">
-        <v>0.2018473632614193</v>
+        <v>0.2349627788858671</v>
       </c>
     </row>
     <row r="257">
@@ -2997,7 +2997,7 @@
         </is>
       </c>
       <c r="B257" t="n">
-        <v>0.06051445365492367</v>
+        <v>0.078240708003736</v>
       </c>
     </row>
     <row r="258">
@@ -3007,7 +3007,7 @@
         </is>
       </c>
       <c r="B258" t="n">
-        <v>0.01074302891758962</v>
+        <v>0.002524908841057994</v>
       </c>
     </row>
     <row r="259">
@@ -3017,7 +3017,7 @@
         </is>
       </c>
       <c r="B259" t="n">
-        <v>0.03776591117759292</v>
+        <v>0.02849391212541904</v>
       </c>
     </row>
     <row r="260">
@@ -3027,7 +3027,7 @@
         </is>
       </c>
       <c r="B260" t="n">
-        <v>0.05986797334998429</v>
+        <v>0.06103389343242571</v>
       </c>
     </row>
     <row r="261">
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="B262" t="n">
-        <v>0.01787032873959218</v>
+        <v>0.02366410110442927</v>
       </c>
     </row>
     <row r="263">
@@ -3057,7 +3057,7 @@
         </is>
       </c>
       <c r="B263" t="n">
-        <v>0.008806673054485892</v>
+        <v>0.01000049861138433</v>
       </c>
     </row>
     <row r="264">
@@ -3067,7 +3067,7 @@
         </is>
       </c>
       <c r="B264" t="n">
-        <v>0.0832586599362679</v>
+        <v>0.05236924977007811</v>
       </c>
     </row>
     <row r="265">
@@ -3077,7 +3077,7 @@
         </is>
       </c>
       <c r="B265" t="n">
-        <v>0.1745684933386115</v>
+        <v>0.1649638807494482</v>
       </c>
     </row>
     <row r="266">
@@ -3087,7 +3087,7 @@
         </is>
       </c>
       <c r="B266" t="n">
-        <v>0.06032287094450588</v>
+        <v>0.01504615548551557</v>
       </c>
     </row>
     <row r="267">
@@ -3097,7 +3097,7 @@
         </is>
       </c>
       <c r="B267" t="n">
-        <v>0.01096193815047545</v>
+        <v>0.0120940250873706</v>
       </c>
     </row>
     <row r="268">
@@ -3107,7 +3107,7 @@
         </is>
       </c>
       <c r="B268" t="n">
-        <v>0.00673332241505014</v>
+        <v>0.00117024875995026</v>
       </c>
     </row>
     <row r="269">
@@ -3117,7 +3117,7 @@
         </is>
       </c>
       <c r="B269" t="n">
-        <v>0.1461666361821978</v>
+        <v>0.1228611762160168</v>
       </c>
     </row>
     <row r="270">
@@ -3127,7 +3127,7 @@
         </is>
       </c>
       <c r="B270" t="n">
-        <v>0.1784037961031667</v>
+        <v>0.1703983613504732</v>
       </c>
     </row>
     <row r="271">
@@ -3137,7 +3137,7 @@
         </is>
       </c>
       <c r="B271" t="n">
-        <v>0.0859197417360181</v>
+        <v>0.0943428421309959</v>
       </c>
     </row>
     <row r="272">
@@ -3147,7 +3147,7 @@
         </is>
       </c>
       <c r="B272" t="n">
-        <v>0.02247387640989053</v>
+        <v>0.01895179081925137</v>
       </c>
     </row>
     <row r="273">
@@ -3157,7 +3157,7 @@
         </is>
       </c>
       <c r="B273" t="n">
-        <v>0.048284810251641</v>
+        <v>0.03619689805278629</v>
       </c>
     </row>
     <row r="274">
@@ -3167,7 +3167,7 @@
         </is>
       </c>
       <c r="B274" t="n">
-        <v>0.01087445104269795</v>
+        <v>0.01147743843727363</v>
       </c>
     </row>
     <row r="275">
@@ -3177,7 +3177,7 @@
         </is>
       </c>
       <c r="B275" t="n">
-        <v>0.06814402541807767</v>
+        <v>0.07442567860624955</v>
       </c>
     </row>
     <row r="276">
@@ -3187,7 +3187,7 @@
         </is>
       </c>
       <c r="B276" t="n">
-        <v>0.01149957158964809</v>
+        <v>0.01050557305630072</v>
       </c>
     </row>
     <row r="277">
@@ -3207,7 +3207,7 @@
         </is>
       </c>
       <c r="B278" t="n">
-        <v>0.02223900251567245</v>
+        <v>0.02113069116950765</v>
       </c>
     </row>
     <row r="279">
@@ -3217,7 +3217,7 @@
         </is>
       </c>
       <c r="B279" t="n">
-        <v>0.05360189023541154</v>
+        <v>0.04400709468640886</v>
       </c>
     </row>
     <row r="280">
@@ -3227,7 +3227,7 @@
         </is>
       </c>
       <c r="B280" t="n">
-        <v>0.01838660126171957</v>
+        <v>0.01918404584213141</v>
       </c>
     </row>
     <row r="281">
@@ -3257,7 +3257,7 @@
         </is>
       </c>
       <c r="B283" t="n">
-        <v>0.000922011006822626</v>
+        <v>0.001234688464506173</v>
       </c>
     </row>
     <row r="284">
@@ -3267,7 +3267,7 @@
         </is>
       </c>
       <c r="B284" t="n">
-        <v>0.02760650897966477</v>
+        <v>0.02534854265330474</v>
       </c>
     </row>
     <row r="285">
@@ -3277,7 +3277,7 @@
         </is>
       </c>
       <c r="B285" t="n">
-        <v>0.02453055465103658</v>
+        <v>0.02997245179063361</v>
       </c>
     </row>
     <row r="286">
@@ -3287,7 +3287,7 @@
         </is>
       </c>
       <c r="B286" t="n">
-        <v>0.0004078333527596192</v>
+        <v>0.001121273742086586</v>
       </c>
     </row>
     <row r="287">
@@ -3297,7 +3297,7 @@
         </is>
       </c>
       <c r="B287" t="n">
-        <v>0.03441236746890665</v>
+        <v>0.02834754599684087</v>
       </c>
     </row>
     <row r="288">
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="B288" t="n">
-        <v>0.1119544988176479</v>
+        <v>0.110691200261492</v>
       </c>
     </row>
     <row r="289">
@@ -3317,7 +3317,7 @@
         </is>
       </c>
       <c r="B289" t="n">
-        <v>0.05285009748933481</v>
+        <v>0.07751364232715698</v>
       </c>
     </row>
     <row r="290">
@@ -3327,7 +3327,7 @@
         </is>
       </c>
       <c r="B290" t="n">
-        <v>0.1382105942005628</v>
+        <v>0.1298813082418485</v>
       </c>
     </row>
     <row r="291">
@@ -3337,7 +3337,7 @@
         </is>
       </c>
       <c r="B291" t="n">
-        <v>0.01232933948175326</v>
+        <v>0.009275633999733615</v>
       </c>
     </row>
     <row r="292">
@@ -3347,7 +3347,7 @@
         </is>
       </c>
       <c r="B292" t="n">
-        <v>0.01210226838256986</v>
+        <v>0.01114768479706786</v>
       </c>
     </row>
     <row r="293">
@@ -3357,7 +3357,7 @@
         </is>
       </c>
       <c r="B293" t="n">
-        <v>0.02898405571244316</v>
+        <v>0.06879347721224269</v>
       </c>
     </row>
     <row r="294">
@@ -3367,7 +3367,7 @@
         </is>
       </c>
       <c r="B294" t="n">
-        <v>0.01877201533960154</v>
+        <v>0.05208210514381306</v>
       </c>
     </row>
     <row r="295">
@@ -3387,7 +3387,7 @@
         </is>
       </c>
       <c r="B296" t="n">
-        <v>0.01587221960279771</v>
+        <v>0.02497671156977996</v>
       </c>
     </row>
     <row r="297">
@@ -3397,7 +3397,7 @@
         </is>
       </c>
       <c r="B297" t="n">
-        <v>0.01138591378975098</v>
+        <v>0.00662374734578946</v>
       </c>
     </row>
     <row r="298">
@@ -3407,7 +3407,7 @@
         </is>
       </c>
       <c r="B298" t="n">
-        <v>0.009260647686040374</v>
+        <v>0.04155087524891863</v>
       </c>
     </row>
     <row r="299">
@@ -3417,7 +3417,7 @@
         </is>
       </c>
       <c r="B299" t="n">
-        <v>0.03821140843509945</v>
+        <v>0.03927233695633622</v>
       </c>
     </row>
     <row r="300">
@@ -3427,7 +3427,7 @@
         </is>
       </c>
       <c r="B300" t="n">
-        <v>0.02132304571013259</v>
+        <v>0.02674929805475001</v>
       </c>
     </row>
     <row r="301">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="B301" t="n">
-        <v>0.1041558103250053</v>
+        <v>0.05414704213581011</v>
       </c>
     </row>
     <row r="302">
@@ -3447,7 +3447,7 @@
         </is>
       </c>
       <c r="B302" t="n">
-        <v>0.02690950303519295</v>
+        <v>0.03270561482269627</v>
       </c>
     </row>
     <row r="303">
@@ -3457,7 +3457,7 @@
         </is>
       </c>
       <c r="B303" t="n">
-        <v>0.01371289459601674</v>
+        <v>0.01645629419455836</v>
       </c>
     </row>
     <row r="304">
@@ -3477,7 +3477,7 @@
         </is>
       </c>
       <c r="B305" t="n">
-        <v>0.06807408929159786</v>
+        <v>0.07202012025369933</v>
       </c>
     </row>
     <row r="306">
@@ -3497,7 +3497,7 @@
         </is>
       </c>
       <c r="B307" t="n">
-        <v>0.02139959606949804</v>
+        <v>0.02003409472976848</v>
       </c>
     </row>
     <row r="308">
@@ -3507,7 +3507,7 @@
         </is>
       </c>
       <c r="B308" t="n">
-        <v>0.01750451324543839</v>
+        <v>0.01615278271895926</v>
       </c>
     </row>
     <row r="309">
@@ -3517,7 +3517,7 @@
         </is>
       </c>
       <c r="B309" t="n">
-        <v>0.008698163220779861</v>
+        <v>0.01699399488760691</v>
       </c>
     </row>
     <row r="310">
@@ -3527,7 +3527,7 @@
         </is>
       </c>
       <c r="B310" t="n">
-        <v>0.1691606877721696</v>
+        <v>0.1157057861923274</v>
       </c>
     </row>
     <row r="311">
@@ -3537,7 +3537,7 @@
         </is>
       </c>
       <c r="B311" t="n">
-        <v>0.0218234608083252</v>
+        <v>0.01506176167940557</v>
       </c>
     </row>
     <row r="312">
@@ -3557,7 +3557,7 @@
         </is>
       </c>
       <c r="B313" t="n">
-        <v>0.03149814814678335</v>
+        <v>0.1260329671690593</v>
       </c>
     </row>
     <row r="314">
@@ -3567,7 +3567,7 @@
         </is>
       </c>
       <c r="B314" t="n">
-        <v>0.1101283961987103</v>
+        <v>0.09229539120648336</v>
       </c>
     </row>
     <row r="315">
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="B315" t="n">
-        <v>0.1472351456348514</v>
+        <v>0.1069855156445302</v>
       </c>
     </row>
     <row r="316">
@@ -3587,7 +3587,7 @@
         </is>
       </c>
       <c r="B316" t="n">
-        <v>0.01536312295933689</v>
+        <v>0.02024690937175482</v>
       </c>
     </row>
     <row r="317">
@@ -3597,7 +3597,7 @@
         </is>
       </c>
       <c r="B317" t="n">
-        <v>0.07662914911835404</v>
+        <v>0.0653954066126647</v>
       </c>
     </row>
     <row r="318">
@@ -3607,7 +3607,7 @@
         </is>
       </c>
       <c r="B318" t="n">
-        <v>0.006933275538818507</v>
+        <v>0.00513757402470809</v>
       </c>
     </row>
     <row r="319">
@@ -3617,7 +3617,7 @@
         </is>
       </c>
       <c r="B319" t="n">
-        <v>0.1133335099844545</v>
+        <v>0.1050553849640236</v>
       </c>
     </row>
     <row r="320">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="B320" t="n">
-        <v>0.04076545777427826</v>
+        <v>0.05623415596691304</v>
       </c>
     </row>
     <row r="321">
@@ -3637,7 +3637,7 @@
         </is>
       </c>
       <c r="B321" t="n">
-        <v>0.02588730559468121</v>
+        <v>0.02490124938569762</v>
       </c>
     </row>
     <row r="322">
@@ -3647,7 +3647,7 @@
         </is>
       </c>
       <c r="B322" t="n">
-        <v>0.03597432030055124</v>
+        <v>0.06271590160406719</v>
       </c>
     </row>
     <row r="323">
@@ -3657,7 +3657,7 @@
         </is>
       </c>
       <c r="B323" t="n">
-        <v>0.001674380822074303</v>
+        <v>0.01800516884226066</v>
       </c>
     </row>
     <row r="324">
@@ -3667,7 +3667,7 @@
         </is>
       </c>
       <c r="B324" t="n">
-        <v>0.03504451705870114</v>
+        <v>0.0248888047878698</v>
       </c>
     </row>
     <row r="325">
@@ -3677,7 +3677,7 @@
         </is>
       </c>
       <c r="B325" t="n">
-        <v>0.06640472937160885</v>
+        <v>0.08382173377029541</v>
       </c>
     </row>
     <row r="326">
@@ -3707,7 +3707,7 @@
         </is>
       </c>
       <c r="B328" t="n">
-        <v>0.01108656240721516</v>
+        <v>0</v>
       </c>
     </row>
     <row r="329">
@@ -3717,7 +3717,7 @@
         </is>
       </c>
       <c r="B329" t="n">
-        <v>0.2116763461485019</v>
+        <v>0.2124707816666457</v>
       </c>
     </row>
     <row r="330">
@@ -3727,7 +3727,7 @@
         </is>
       </c>
       <c r="B330" t="n">
-        <v>0.0293445305991972</v>
+        <v>0.01525688063724863</v>
       </c>
     </row>
     <row r="331">
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="B331" t="n">
-        <v>0.04975267303970775</v>
+        <v>0.05634863913722681</v>
       </c>
     </row>
     <row r="332">
@@ -3747,7 +3747,7 @@
         </is>
       </c>
       <c r="B332" t="n">
-        <v>0.01124497071349209</v>
+        <v>0.01008702872139817</v>
       </c>
     </row>
     <row r="333">
@@ -3757,7 +3757,7 @@
         </is>
       </c>
       <c r="B333" t="n">
-        <v>0.1342000951647992</v>
+        <v>0.1328508612498616</v>
       </c>
     </row>
     <row r="334">
@@ -3767,7 +3767,7 @@
         </is>
       </c>
       <c r="B334" t="n">
-        <v>0.08155459786292421</v>
+        <v>0.07364403945264811</v>
       </c>
     </row>
     <row r="335">
@@ -3777,7 +3777,7 @@
         </is>
       </c>
       <c r="B335" t="n">
-        <v>0.008228992236381204</v>
+        <v>0.009074936433832457</v>
       </c>
     </row>
     <row r="336">
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="B336" t="n">
-        <v>0.1253489782277191</v>
+        <v>0.1135113547492278</v>
       </c>
     </row>
     <row r="337">
@@ -3797,7 +3797,7 @@
         </is>
       </c>
       <c r="B337" t="n">
-        <v>0.01378463020892199</v>
+        <v>0.01450903023908238</v>
       </c>
     </row>
     <row r="338">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="B338" t="n">
-        <v>0.0844449807631364</v>
+        <v>0.1127715756809027</v>
       </c>
     </row>
     <row r="339">
@@ -3817,7 +3817,7 @@
         </is>
       </c>
       <c r="B339" t="n">
-        <v>0.06349294739547824</v>
+        <v>0.06931176343385839</v>
       </c>
     </row>
     <row r="340">
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="B340" t="n">
-        <v>0.002078366459349609</v>
+        <v>0.03620226527034785</v>
       </c>
     </row>
     <row r="341">
@@ -3837,7 +3837,7 @@
         </is>
       </c>
       <c r="B341" t="n">
-        <v>0.06338777926465497</v>
+        <v>0.07094831250378925</v>
       </c>
     </row>
     <row r="342">
@@ -3847,7 +3847,7 @@
         </is>
       </c>
       <c r="B342" t="n">
-        <v>0.04745421554878846</v>
+        <v>0.05637373168408395</v>
       </c>
     </row>
     <row r="343">
@@ -3857,7 +3857,7 @@
         </is>
       </c>
       <c r="B343" t="n">
-        <v>0.08266993047695566</v>
+        <v>0.08472718979844121</v>
       </c>
     </row>
     <row r="344">
@@ -3867,7 +3867,7 @@
         </is>
       </c>
       <c r="B344" t="n">
-        <v>0.12311593210432</v>
+        <v>0.09464494285908849</v>
       </c>
     </row>
     <row r="345">
@@ -3877,7 +3877,7 @@
         </is>
       </c>
       <c r="B345" t="n">
-        <v>0.06859848760106245</v>
+        <v>0.07117803565951419</v>
       </c>
     </row>
     <row r="346">
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="B346" t="n">
-        <v>0.06491061009732664</v>
+        <v>0.06056331193857192</v>
       </c>
     </row>
     <row r="347">
@@ -3897,7 +3897,7 @@
         </is>
       </c>
       <c r="B347" t="n">
-        <v>0.03350585731974914</v>
+        <v>0.040539422311269</v>
       </c>
     </row>
     <row r="348">
@@ -3907,7 +3907,7 @@
         </is>
       </c>
       <c r="B348" t="n">
-        <v>0.06812334256137063</v>
+        <v>0.04498644663176957</v>
       </c>
     </row>
     <row r="349">
@@ -3917,7 +3917,7 @@
         </is>
       </c>
       <c r="B349" t="n">
-        <v>0.02454960140603352</v>
+        <v>0.02520205441032976</v>
       </c>
     </row>
     <row r="350">
@@ -3927,7 +3927,7 @@
         </is>
       </c>
       <c r="B350" t="n">
-        <v>0.08057664156923786</v>
+        <v>0.06040955087562747</v>
       </c>
     </row>
     <row r="351">
@@ -3937,7 +3937,7 @@
         </is>
       </c>
       <c r="B351" t="n">
-        <v>0.006010642564702054</v>
+        <v>0.005290774738310428</v>
       </c>
     </row>
     <row r="352">
@@ -3947,7 +3947,7 @@
         </is>
       </c>
       <c r="B352" t="n">
-        <v>0.03584793795630037</v>
+        <v>0.04412731419419769</v>
       </c>
     </row>
     <row r="353">
@@ -3957,7 +3957,7 @@
         </is>
       </c>
       <c r="B353" t="n">
-        <v>0.006010210259573438</v>
+        <v>0.008868850189196425</v>
       </c>
     </row>
     <row r="354">
@@ -3967,7 +3967,7 @@
         </is>
       </c>
       <c r="B354" t="n">
-        <v>0.04116460018555546</v>
+        <v>0.04150544123262793</v>
       </c>
     </row>
     <row r="355">
@@ -3977,7 +3977,7 @@
         </is>
       </c>
       <c r="B355" t="n">
-        <v>0.01969842399537648</v>
+        <v>0.04102111962119464</v>
       </c>
     </row>
     <row r="356">
@@ -3987,7 +3987,7 @@
         </is>
       </c>
       <c r="B356" t="n">
-        <v>0.03267419413007259</v>
+        <v>0.02997587631389834</v>
       </c>
     </row>
     <row r="357">
@@ -3997,7 +3997,7 @@
         </is>
       </c>
       <c r="B357" t="n">
-        <v>0.03915825157895578</v>
+        <v>0.02035865701100629</v>
       </c>
     </row>
     <row r="358">
@@ -4007,7 +4007,7 @@
         </is>
       </c>
       <c r="B358" t="n">
-        <v>0.06735480189750921</v>
+        <v>0.0639196174299269</v>
       </c>
     </row>
     <row r="359">
@@ -4017,7 +4017,7 @@
         </is>
       </c>
       <c r="B359" t="n">
-        <v>0.03453326150916948</v>
+        <v>0.06254129728913357</v>
       </c>
     </row>
     <row r="360">
@@ -4027,7 +4027,7 @@
         </is>
       </c>
       <c r="B360" t="n">
-        <v>0.005901823471414987</v>
+        <v>0.005879528775967406</v>
       </c>
     </row>
     <row r="361">
@@ -4037,7 +4037,7 @@
         </is>
       </c>
       <c r="B361" t="n">
-        <v>0.08079168727349981</v>
+        <v>0.0735330335812457</v>
       </c>
     </row>
     <row r="362">
@@ -4057,7 +4057,7 @@
         </is>
       </c>
       <c r="B363" t="n">
-        <v>0.04745978726905963</v>
+        <v>0.03917487426568857</v>
       </c>
     </row>
     <row r="364">
@@ -4067,7 +4067,7 @@
         </is>
       </c>
       <c r="B364" t="n">
-        <v>0.05406496127810773</v>
+        <v>0.05872119762099575</v>
       </c>
     </row>
     <row r="365">
@@ -4077,7 +4077,7 @@
         </is>
       </c>
       <c r="B365" t="n">
-        <v>0.06034747071649875</v>
+        <v>0.03842026736970446</v>
       </c>
     </row>
     <row r="366">
@@ -4087,7 +4087,7 @@
         </is>
       </c>
       <c r="B366" t="n">
-        <v>0.05439573536445213</v>
+        <v>0.0678339147642909</v>
       </c>
     </row>
     <row r="367">
@@ -4097,7 +4097,7 @@
         </is>
       </c>
       <c r="B367" t="n">
-        <v>0.03615238807071779</v>
+        <v>0.03362689509841292</v>
       </c>
     </row>
     <row r="368">
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="B368" t="n">
-        <v>0.02902669378639813</v>
+        <v>0.01881022853314103</v>
       </c>
     </row>
     <row r="369">
@@ -4117,7 +4117,7 @@
         </is>
       </c>
       <c r="B369" t="n">
-        <v>0.03275570987784361</v>
+        <v>0.03686079038893292</v>
       </c>
     </row>
     <row r="370">
@@ -4127,7 +4127,7 @@
         </is>
       </c>
       <c r="B370" t="n">
-        <v>0.02384193235823052</v>
+        <v>0.0325900630058553</v>
       </c>
     </row>
     <row r="371">
@@ -4137,7 +4137,7 @@
         </is>
       </c>
       <c r="B371" t="n">
-        <v>0.01966986070801824</v>
+        <v>0.01468677523370061</v>
       </c>
     </row>
     <row r="372">
@@ -4147,7 +4147,7 @@
         </is>
       </c>
       <c r="B372" t="n">
-        <v>0.06785485368617596</v>
+        <v>0.06850876531993554</v>
       </c>
     </row>
     <row r="373">
@@ -4157,7 +4157,7 @@
         </is>
       </c>
       <c r="B373" t="n">
-        <v>0.1494155600459534</v>
+        <v>0.04178632969557725</v>
       </c>
     </row>
     <row r="374">
@@ -4167,7 +4167,7 @@
         </is>
       </c>
       <c r="B374" t="n">
-        <v>0.03685646497169795</v>
+        <v>0.01980930512724971</v>
       </c>
     </row>
     <row r="375">
@@ -4177,7 +4177,7 @@
         </is>
       </c>
       <c r="B375" t="n">
-        <v>0.06948265554593802</v>
+        <v>0.06615267239801938</v>
       </c>
     </row>
     <row r="376">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="B376" t="n">
-        <v>0.09575939687958168</v>
+        <v>0.08572949288837566</v>
       </c>
     </row>
     <row r="377">
@@ -4197,7 +4197,7 @@
         </is>
       </c>
       <c r="B377" t="n">
-        <v>0.08537720453920912</v>
+        <v>0.07726962547445927</v>
       </c>
     </row>
     <row r="378">
@@ -4207,7 +4207,7 @@
         </is>
       </c>
       <c r="B378" t="n">
-        <v>0.04318699484658538</v>
+        <v>0.07848995622673263</v>
       </c>
     </row>
     <row r="379">
@@ -4217,7 +4217,7 @@
         </is>
       </c>
       <c r="B379" t="n">
-        <v>0.02618719576779175</v>
+        <v>0.03283187844152755</v>
       </c>
     </row>
     <row r="380">
@@ -4227,7 +4227,7 @@
         </is>
       </c>
       <c r="B380" t="n">
-        <v>0.01921626632715876</v>
+        <v>0.01630105801451325</v>
       </c>
     </row>
     <row r="381">
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="B381" t="n">
-        <v>0.08266124796390574</v>
+        <v>0.07735993425830344</v>
       </c>
     </row>
     <row r="382">
@@ -4247,7 +4247,7 @@
         </is>
       </c>
       <c r="B382" t="n">
-        <v>0.02963853491817214</v>
+        <v>0.02349541226677775</v>
       </c>
     </row>
     <row r="383">
@@ -4257,7 +4257,7 @@
         </is>
       </c>
       <c r="B383" t="n">
-        <v>0.07776287093943053</v>
+        <v>0.08526170027662372</v>
       </c>
     </row>
     <row r="384">
@@ -4267,7 +4267,7 @@
         </is>
       </c>
       <c r="B384" t="n">
-        <v>0.05464020780094837</v>
+        <v>0.04805171826957261</v>
       </c>
     </row>
     <row r="385">
@@ -4277,7 +4277,7 @@
         </is>
       </c>
       <c r="B385" t="n">
-        <v>0.01342732200607956</v>
+        <v>0.01156870758682783</v>
       </c>
     </row>
     <row r="386">
@@ -4287,7 +4287,7 @@
         </is>
       </c>
       <c r="B386" t="n">
-        <v>0.06499408073386859</v>
+        <v>0.08872569844900233</v>
       </c>
     </row>
     <row r="387">
@@ -4297,7 +4297,7 @@
         </is>
       </c>
       <c r="B387" t="n">
-        <v>0.00486853421201709</v>
+        <v>0.00202253709181905</v>
       </c>
     </row>
     <row r="388">
@@ -4307,7 +4307,7 @@
         </is>
       </c>
       <c r="B388" t="n">
-        <v>0.03779416222617059</v>
+        <v>0.02973838202537243</v>
       </c>
     </row>
     <row r="389">
@@ -4317,7 +4317,7 @@
         </is>
       </c>
       <c r="B389" t="n">
-        <v>0.05358575687764511</v>
+        <v>0.05672129160072317</v>
       </c>
     </row>
     <row r="390">
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="B390" t="n">
-        <v>0.06343709849043805</v>
+        <v>0.06065942869612908</v>
       </c>
     </row>
     <row r="391">
@@ -4337,7 +4337,7 @@
         </is>
       </c>
       <c r="B391" t="n">
-        <v>0.007154695516200115</v>
+        <v>0</v>
       </c>
     </row>
     <row r="392">
@@ -4347,7 +4347,7 @@
         </is>
       </c>
       <c r="B392" t="n">
-        <v>0.1149204363981941</v>
+        <v>0.06050474033473392</v>
       </c>
     </row>
     <row r="393">
@@ -4357,7 +4357,7 @@
         </is>
       </c>
       <c r="B393" t="n">
-        <v>0.1024996564881981</v>
+        <v>0.1241970466354477</v>
       </c>
     </row>
     <row r="394">
@@ -4367,7 +4367,7 @@
         </is>
       </c>
       <c r="B394" t="n">
-        <v>0.03665251396997309</v>
+        <v>0.03442121332909014</v>
       </c>
     </row>
     <row r="395">
@@ -4377,7 +4377,7 @@
         </is>
       </c>
       <c r="B395" t="n">
-        <v>0.01278057372072088</v>
+        <v>0.01249435837824776</v>
       </c>
     </row>
     <row r="396">
@@ -4387,7 +4387,7 @@
         </is>
       </c>
       <c r="B396" t="n">
-        <v>0.04221004964323183</v>
+        <v>0.04033653770714933</v>
       </c>
     </row>
     <row r="397">
@@ -4397,7 +4397,7 @@
         </is>
       </c>
       <c r="B397" t="n">
-        <v>0.03672330313368032</v>
+        <v>0.05707919247232507</v>
       </c>
     </row>
     <row r="398">
@@ -4407,7 +4407,7 @@
         </is>
       </c>
       <c r="B398" t="n">
-        <v>0.05398139916068693</v>
+        <v>0.07198050965878032</v>
       </c>
     </row>
     <row r="399">
@@ -4417,7 +4417,7 @@
         </is>
       </c>
       <c r="B399" t="n">
-        <v>0.04651399192908533</v>
+        <v>0.04622544518622129</v>
       </c>
     </row>
     <row r="400">
@@ -4427,7 +4427,7 @@
         </is>
       </c>
       <c r="B400" t="n">
-        <v>0.1551946649665741</v>
+        <v>0.1455009395136745</v>
       </c>
     </row>
     <row r="401">
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="B401" t="n">
-        <v>0.02428856141626288</v>
+        <v>0.03730794110433089</v>
       </c>
     </row>
     <row r="402">
@@ -4447,7 +4447,7 @@
         </is>
       </c>
       <c r="B402" t="n">
-        <v>0.005867644182233529</v>
+        <v>0.004137402676073904</v>
       </c>
     </row>
     <row r="403">
@@ -4457,7 +4457,7 @@
         </is>
       </c>
       <c r="B403" t="n">
-        <v>0.04997949664914185</v>
+        <v>0.0567110412144828</v>
       </c>
     </row>
     <row r="404">
@@ -4467,7 +4467,7 @@
         </is>
       </c>
       <c r="B404" t="n">
-        <v>0.03493004111519965</v>
+        <v>0.04392991611130533</v>
       </c>
     </row>
     <row r="405">
@@ -4487,7 +4487,7 @@
         </is>
       </c>
       <c r="B406" t="n">
-        <v>0.07990711520131671</v>
+        <v>0.1007106339717374</v>
       </c>
     </row>
     <row r="407">
@@ -4497,7 +4497,7 @@
         </is>
       </c>
       <c r="B407" t="n">
-        <v>0.0672996350088472</v>
+        <v>0.04980754840763146</v>
       </c>
     </row>
     <row r="408">
@@ -4507,7 +4507,7 @@
         </is>
       </c>
       <c r="B408" t="n">
-        <v>0.03668604196705</v>
+        <v>0.03091320480509759</v>
       </c>
     </row>
     <row r="409">
@@ -4517,7 +4517,7 @@
         </is>
       </c>
       <c r="B409" t="n">
-        <v>0.1596822683927369</v>
+        <v>0.170542163116391</v>
       </c>
     </row>
     <row r="410">
@@ -4527,7 +4527,7 @@
         </is>
       </c>
       <c r="B410" t="n">
-        <v>0.0365785383332182</v>
+        <v>0.03586231350699736</v>
       </c>
     </row>
     <row r="411">
@@ -4537,7 +4537,7 @@
         </is>
       </c>
       <c r="B411" t="n">
-        <v>0.04195563412326741</v>
+        <v>0.03190853524514001</v>
       </c>
     </row>
     <row r="412">
@@ -4547,7 +4547,7 @@
         </is>
       </c>
       <c r="B412" t="n">
-        <v>0.04860276415488605</v>
+        <v>0.04221122876951438</v>
       </c>
     </row>
     <row r="413">
@@ -4557,7 +4557,7 @@
         </is>
       </c>
       <c r="B413" t="n">
-        <v>0.1098060348427177</v>
+        <v>0.08085374146986558</v>
       </c>
     </row>
     <row r="414">
@@ -4567,7 +4567,7 @@
         </is>
       </c>
       <c r="B414" t="n">
-        <v>0.07472706073561107</v>
+        <v>0.0745374449339207</v>
       </c>
     </row>
     <row r="415">
@@ -4577,7 +4577,7 @@
         </is>
       </c>
       <c r="B415" t="n">
-        <v>0.05129154784918618</v>
+        <v>0.0749862026991225</v>
       </c>
     </row>
     <row r="416">
@@ -4587,7 +4587,7 @@
         </is>
       </c>
       <c r="B416" t="n">
-        <v>0.1920775682080222</v>
+        <v>0.170816336506787</v>
       </c>
     </row>
     <row r="417">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="B418" t="n">
-        <v>0.1500959862187307</v>
+        <v>0.1401376467401358</v>
       </c>
     </row>
     <row r="419">
@@ -4617,7 +4617,7 @@
         </is>
       </c>
       <c r="B419" t="n">
-        <v>0.08814824113186194</v>
+        <v>0.1208993755062686</v>
       </c>
     </row>
     <row r="420">
@@ -4627,7 +4627,7 @@
         </is>
       </c>
       <c r="B420" t="n">
-        <v>0.0549269269497904</v>
+        <v>0.05790898512901928</v>
       </c>
     </row>
     <row r="421">
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="B421" t="n">
-        <v>0.04201715083117184</v>
+        <v>0.03914601787808899</v>
       </c>
     </row>
     <row r="422">
@@ -4647,7 +4647,7 @@
         </is>
       </c>
       <c r="B422" t="n">
-        <v>0.1080208430445942</v>
+        <v>0.1064355821034391</v>
       </c>
     </row>
     <row r="423">
@@ -4657,7 +4657,7 @@
         </is>
       </c>
       <c r="B423" t="n">
-        <v>0.00542379555915343</v>
+        <v>0.007076932147342962</v>
       </c>
     </row>
     <row r="424">
@@ -4667,7 +4667,7 @@
         </is>
       </c>
       <c r="B424" t="n">
-        <v>0.02312068755291702</v>
+        <v>0.01279053605784932</v>
       </c>
     </row>
     <row r="425">
@@ -4677,7 +4677,7 @@
         </is>
       </c>
       <c r="B425" t="n">
-        <v>0.196144396323476</v>
+        <v>0.2271200985034241</v>
       </c>
     </row>
     <row r="426">
@@ -4687,7 +4687,7 @@
         </is>
       </c>
       <c r="B426" t="n">
-        <v>0.05577066807048062</v>
+        <v>0.08310625481653436</v>
       </c>
     </row>
     <row r="427">
@@ -4697,7 +4697,7 @@
         </is>
       </c>
       <c r="B427" t="n">
-        <v>0.04220241097928253</v>
+        <v>0.0411543741013236</v>
       </c>
     </row>
     <row r="428">
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="B428" t="n">
-        <v>0.02699025924473803</v>
+        <v>0.04325627946376798</v>
       </c>
     </row>
     <row r="429">
@@ -4717,7 +4717,7 @@
         </is>
       </c>
       <c r="B429" t="n">
-        <v>0.03735239668871349</v>
+        <v>0.03826800756075917</v>
       </c>
     </row>
     <row r="430">
@@ -4727,7 +4727,7 @@
         </is>
       </c>
       <c r="B430" t="n">
-        <v>0.02130323029828483</v>
+        <v>0.03243044134774069</v>
       </c>
     </row>
     <row r="431">
@@ -4737,7 +4737,7 @@
         </is>
       </c>
       <c r="B431" t="n">
-        <v>0.05691786910011573</v>
+        <v>0.1068664959242878</v>
       </c>
     </row>
     <row r="432">
@@ -4747,7 +4747,7 @@
         </is>
       </c>
       <c r="B432" t="n">
-        <v>0.04916602846263691</v>
+        <v>0.06610968980699627</v>
       </c>
     </row>
     <row r="433">
@@ -4757,7 +4757,7 @@
         </is>
       </c>
       <c r="B433" t="n">
-        <v>0.02437796569368983</v>
+        <v>0.01815520024188962</v>
       </c>
     </row>
     <row r="434">
@@ -4767,7 +4767,7 @@
         </is>
       </c>
       <c r="B434" t="n">
-        <v>0.02398803396298077</v>
+        <v>0.03569267636333387</v>
       </c>
     </row>
     <row r="435">
@@ -4777,7 +4777,7 @@
         </is>
       </c>
       <c r="B435" t="n">
-        <v>0.0243580891927604</v>
+        <v>0.02077601725264858</v>
       </c>
     </row>
     <row r="436">
@@ -4787,7 +4787,7 @@
         </is>
       </c>
       <c r="B436" t="n">
-        <v>0.05252039347126983</v>
+        <v>0.05023407113440044</v>
       </c>
     </row>
     <row r="437">
@@ -4797,7 +4797,7 @@
         </is>
       </c>
       <c r="B437" t="n">
-        <v>0.05640050670182691</v>
+        <v>0.04840980553372708</v>
       </c>
     </row>
     <row r="438">
@@ -4807,7 +4807,7 @@
         </is>
       </c>
       <c r="B438" t="n">
-        <v>0.01797439942057934</v>
+        <v>0.01651538769338957</v>
       </c>
     </row>
     <row r="439">
@@ -4827,7 +4827,7 @@
         </is>
       </c>
       <c r="B440" t="n">
-        <v>0.08487647897626631</v>
+        <v>0.09072812455627602</v>
       </c>
     </row>
     <row r="441">
@@ -4837,7 +4837,7 @@
         </is>
       </c>
       <c r="B441" t="n">
-        <v>0.05320056546039346</v>
+        <v>0.1021367683433411</v>
       </c>
     </row>
     <row r="442">
@@ -4847,7 +4847,7 @@
         </is>
       </c>
       <c r="B442" t="n">
-        <v>0.07326729615564398</v>
+        <v>0.07417126704692209</v>
       </c>
     </row>
     <row r="443">
@@ -4857,7 +4857,7 @@
         </is>
       </c>
       <c r="B443" t="n">
-        <v>0.1010268128813359</v>
+        <v>0.09649609211260024</v>
       </c>
     </row>
     <row r="444">
@@ -4867,7 +4867,7 @@
         </is>
       </c>
       <c r="B444" t="n">
-        <v>0.07207213211671809</v>
+        <v>0.06681914446810289</v>
       </c>
     </row>
     <row r="445">
@@ -4877,7 +4877,7 @@
         </is>
       </c>
       <c r="B445" t="n">
-        <v>0.1353448830756515</v>
+        <v>0.08881926626663972</v>
       </c>
     </row>
     <row r="446">
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="B446" t="n">
-        <v>0.02927677285647271</v>
+        <v>0.03148275201886713</v>
       </c>
     </row>
     <row r="447">
@@ -4897,7 +4897,7 @@
         </is>
       </c>
       <c r="B447" t="n">
-        <v>0.1404322001237433</v>
+        <v>0.1295668833727625</v>
       </c>
     </row>
     <row r="448">
@@ -4907,7 +4907,7 @@
         </is>
       </c>
       <c r="B448" t="n">
-        <v>0.02620785955628757</v>
+        <v>0.02009751236002226</v>
       </c>
     </row>
     <row r="449">
@@ -4917,7 +4917,7 @@
         </is>
       </c>
       <c r="B449" t="n">
-        <v>0.008386633605510037</v>
+        <v>0.0231454672107667</v>
       </c>
     </row>
     <row r="450">
@@ -4927,7 +4927,7 @@
         </is>
       </c>
       <c r="B450" t="n">
-        <v>0.00751735826362692</v>
+        <v>0.00802076655228327</v>
       </c>
     </row>
     <row r="451">
@@ -4947,7 +4947,7 @@
         </is>
       </c>
       <c r="B452" t="n">
-        <v>0.0283128596587589</v>
+        <v>0.03117593725247008</v>
       </c>
     </row>
     <row r="453">
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="B453" t="n">
-        <v>0.03029449572237806</v>
+        <v>0.02498827424486637</v>
       </c>
     </row>
     <row r="454">
@@ -4967,7 +4967,7 @@
         </is>
       </c>
       <c r="B454" t="n">
-        <v>0.05508269973084551</v>
+        <v>0.03721358890545495</v>
       </c>
     </row>
     <row r="455">
@@ -4977,7 +4977,7 @@
         </is>
       </c>
       <c r="B455" t="n">
-        <v>0.01484906743340088</v>
+        <v>0.01167591879100291</v>
       </c>
     </row>
     <row r="456">
@@ -4987,7 +4987,7 @@
         </is>
       </c>
       <c r="B456" t="n">
-        <v>0.08894250230648726</v>
+        <v>0.05046711237522354</v>
       </c>
     </row>
     <row r="457">
@@ -4997,7 +4997,7 @@
         </is>
       </c>
       <c r="B457" t="n">
-        <v>0.07665156726675139</v>
+        <v>0.06645756234588666</v>
       </c>
     </row>
     <row r="458">
@@ -5007,7 +5007,7 @@
         </is>
       </c>
       <c r="B458" t="n">
-        <v>0.05478537074205326</v>
+        <v>0.05483843587630544</v>
       </c>
     </row>
     <row r="459">
@@ -5017,7 +5017,7 @@
         </is>
       </c>
       <c r="B459" t="n">
-        <v>0.1038189715725248</v>
+        <v>0.1102505373600981</v>
       </c>
     </row>
     <row r="460">
@@ -5027,7 +5027,7 @@
         </is>
       </c>
       <c r="B460" t="n">
-        <v>0.07524150614978352</v>
+        <v>0.05427396233642125</v>
       </c>
     </row>
     <row r="461">
@@ -5037,7 +5037,7 @@
         </is>
       </c>
       <c r="B461" t="n">
-        <v>0.06885821751346737</v>
+        <v>0.1004835743790337</v>
       </c>
     </row>
     <row r="462">
@@ -5047,7 +5047,7 @@
         </is>
       </c>
       <c r="B462" t="n">
-        <v>0.03160929222300431</v>
+        <v>0.04285373954713621</v>
       </c>
     </row>
     <row r="463">
@@ -5057,7 +5057,7 @@
         </is>
       </c>
       <c r="B463" t="n">
-        <v>0.02852574714306402</v>
+        <v>0.02422046720585325</v>
       </c>
     </row>
     <row r="464">
@@ -5067,7 +5067,7 @@
         </is>
       </c>
       <c r="B464" t="n">
-        <v>0.03749201337252011</v>
+        <v>0.0379445910890053</v>
       </c>
     </row>
     <row r="465">
@@ -5077,7 +5077,7 @@
         </is>
       </c>
       <c r="B465" t="n">
-        <v>0.008760824318305828</v>
+        <v>0.1202298702688091</v>
       </c>
     </row>
     <row r="466">
@@ -5097,7 +5097,7 @@
         </is>
       </c>
       <c r="B467" t="n">
-        <v>0.02603168218139511</v>
+        <v>0.0227543418277264</v>
       </c>
     </row>
     <row r="468">
@@ -5107,7 +5107,7 @@
         </is>
       </c>
       <c r="B468" t="n">
-        <v>0.03235068616437</v>
+        <v>0.03987748029888281</v>
       </c>
     </row>
     <row r="469">
@@ -5117,7 +5117,7 @@
         </is>
       </c>
       <c r="B469" t="n">
-        <v>0.02859271991903117</v>
+        <v>0.03045787424384923</v>
       </c>
     </row>
     <row r="470">
@@ -5127,7 +5127,7 @@
         </is>
       </c>
       <c r="B470" t="n">
-        <v>0.01085857546075812</v>
+        <v>0.1049263389077578</v>
       </c>
     </row>
     <row r="471">
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="B471" t="n">
-        <v>0.05147535987139785</v>
+        <v>0.04231565509534749</v>
       </c>
     </row>
     <row r="472">
@@ -5147,7 +5147,7 @@
         </is>
       </c>
       <c r="B472" t="n">
-        <v>0.01139209581097198</v>
+        <v>0.0140055669097524</v>
       </c>
     </row>
     <row r="473">
@@ -5157,7 +5157,7 @@
         </is>
       </c>
       <c r="B473" t="n">
-        <v>0.08558911648133592</v>
+        <v>0.07063793721480109</v>
       </c>
     </row>
     <row r="474">
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="B474" t="n">
-        <v>0.04663901395111954</v>
+        <v>0.05644119597160523</v>
       </c>
     </row>
     <row r="475">
@@ -5177,7 +5177,7 @@
         </is>
       </c>
       <c r="B475" t="n">
-        <v>0.1216758661249713</v>
+        <v>0.04241822091016732</v>
       </c>
     </row>
     <row r="476">
@@ -5187,7 +5187,7 @@
         </is>
       </c>
       <c r="B476" t="n">
-        <v>0.06388580509045706</v>
+        <v>0.0555092076622826</v>
       </c>
     </row>
     <row r="477">
@@ -5197,7 +5197,7 @@
         </is>
       </c>
       <c r="B477" t="n">
-        <v>0.0182955073515384</v>
+        <v>0.01776935342935605</v>
       </c>
     </row>
     <row r="478">
@@ -5207,7 +5207,7 @@
         </is>
       </c>
       <c r="B478" t="n">
-        <v>0.04898422112532345</v>
+        <v>0.05454941414851559</v>
       </c>
     </row>
     <row r="479">
@@ -5217,7 +5217,7 @@
         </is>
       </c>
       <c r="B479" t="n">
-        <v>0.05900186351064597</v>
+        <v>0.04783854796597101</v>
       </c>
     </row>
     <row r="480">
@@ -5237,7 +5237,7 @@
         </is>
       </c>
       <c r="B481" t="n">
-        <v>0.03030409119691591</v>
+        <v>0.03751778264448626</v>
       </c>
     </row>
     <row r="482">
@@ -5247,7 +5247,7 @@
         </is>
       </c>
       <c r="B482" t="n">
-        <v>0.04270164810928562</v>
+        <v>0.04176975245046916</v>
       </c>
     </row>
     <row r="483">
@@ -5257,7 +5257,7 @@
         </is>
       </c>
       <c r="B483" t="n">
-        <v>0.01303938963858505</v>
+        <v>0.01908344993799694</v>
       </c>
     </row>
     <row r="484">
@@ -5267,7 +5267,7 @@
         </is>
       </c>
       <c r="B484" t="n">
-        <v>0.02403490064182073</v>
+        <v>0.0237186579844877</v>
       </c>
     </row>
     <row r="485">
@@ -5277,7 +5277,7 @@
         </is>
       </c>
       <c r="B485" t="n">
-        <v>0.06910522726778127</v>
+        <v>0.0448751499103594</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update README and evaluation scripts for Design2Code-18B-V0. Add summary statistics for IOU scores, improve bounding box extraction logic, and adjust output paths for evaluation results. Update Excel reports for consistency across metrics.
</commit_message>
<xml_diff>
--- a/design2code-18b-v0/evaluation_results/iou_scores.xlsx
+++ b/design2code-18b-v0/evaluation_results/iou_scores.xlsx
@@ -447,7 +447,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.05134755444786486</v>
+        <v>0.1138648336165427</v>
       </c>
     </row>
     <row r="3">
@@ -457,7 +457,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1014903897643338</v>
+        <v>0.1354662536361466</v>
       </c>
     </row>
     <row r="4">
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.04674590514765344</v>
+        <v>0.2016148943678126</v>
       </c>
     </row>
     <row r="5">
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.06968615415455512</v>
+        <v>0.129584676883819</v>
       </c>
     </row>
     <row r="6">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.1024301991291484</v>
+        <v>0.1605103006405593</v>
       </c>
     </row>
     <row r="7">
@@ -497,7 +497,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.03989048530678253</v>
+        <v>0.1444628582085171</v>
       </c>
     </row>
     <row r="8">
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.02319126266457221</v>
+        <v>0.1385600683050163</v>
       </c>
     </row>
     <row r="9">
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.07140766377714482</v>
+        <v>0.1520550872808012</v>
       </c>
     </row>
     <row r="10">
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.00358778480567726</v>
+        <v>0.02093538906170793</v>
       </c>
     </row>
     <row r="11">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0261665672062389</v>
+        <v>0.07228881650592696</v>
       </c>
     </row>
     <row r="12">
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.01620734167652354</v>
+        <v>0.03615602813550933</v>
       </c>
     </row>
     <row r="13">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1796640291774187</v>
+        <v>0.1993030891146629</v>
       </c>
     </row>
     <row r="14">
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.02043242658813808</v>
+        <v>0.05291645032957863</v>
       </c>
     </row>
     <row r="16">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.04396106864263459</v>
+        <v>0.1478696590110478</v>
       </c>
     </row>
     <row r="17">
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>0.06187604826880731</v>
       </c>
     </row>
     <row r="18">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.0829898708523799</v>
+        <v>0.1413125840677278</v>
       </c>
     </row>
     <row r="19">
@@ -617,7 +617,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.07597697694436852</v>
+        <v>0.1026543143428994</v>
       </c>
     </row>
     <row r="20">
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.05142092703225967</v>
+        <v>0.1111934351850598</v>
       </c>
     </row>
     <row r="21">
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.03786582545329591</v>
+        <v>0.1231195014560275</v>
       </c>
     </row>
     <row r="22">
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.101170661784897</v>
+        <v>0.1540419954691092</v>
       </c>
     </row>
     <row r="23">
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.07101726986760931</v>
+        <v>0.1106469751694115</v>
       </c>
     </row>
     <row r="24">
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0</v>
+        <v>0.1154127729594895</v>
       </c>
     </row>
     <row r="25">
@@ -677,7 +677,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.111494405096134</v>
+        <v>0.2113627381714331</v>
       </c>
     </row>
     <row r="26">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.09164505162350194</v>
+        <v>0.1137817406422002</v>
       </c>
     </row>
     <row r="27">
@@ -697,7 +697,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.006551186464030947</v>
+        <v>0.1109414990181995</v>
       </c>
     </row>
     <row r="28">
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.0128677380322735</v>
+        <v>0.0858908944687978</v>
       </c>
     </row>
     <row r="29">
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.02691094067499085</v>
+        <v>0.05939677427386816</v>
       </c>
     </row>
     <row r="30">
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.07589092132146001</v>
+        <v>0.1505541213337465</v>
       </c>
     </row>
     <row r="31">
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.05038301466842739</v>
+        <v>0.1108737757446568</v>
       </c>
     </row>
     <row r="32">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.01263001720743036</v>
+        <v>0.106198399840375</v>
       </c>
     </row>
     <row r="33">
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0.05986420688992944</v>
+        <v>0.1136864031141114</v>
       </c>
     </row>
     <row r="34">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.0244275354443925</v>
+        <v>0.1212352326725309</v>
       </c>
     </row>
     <row r="35">
@@ -777,7 +777,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.01833584596208234</v>
+        <v>0.1435204998242438</v>
       </c>
     </row>
     <row r="36">
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.02782230638329327</v>
+        <v>0.08097165659193492</v>
       </c>
     </row>
     <row r="37">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.2360276610810076</v>
+        <v>0.3080455382780335</v>
       </c>
     </row>
     <row r="38">
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.1074123602167478</v>
+        <v>0.1469350602702404</v>
       </c>
     </row>
     <row r="39">
@@ -817,7 +817,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.04354998874612579</v>
+        <v>0.1959963022516296</v>
       </c>
     </row>
     <row r="40">
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.007661221799391069</v>
+        <v>0.06189306388777627</v>
       </c>
     </row>
     <row r="41">
@@ -837,7 +837,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.1227554565921946</v>
+        <v>0.1495436331770821</v>
       </c>
     </row>
     <row r="42">
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.1095461288194616</v>
+        <v>0.1807179834229725</v>
       </c>
     </row>
     <row r="43">
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.07609670903245533</v>
+        <v>0.1242155684614153</v>
       </c>
     </row>
     <row r="44">
@@ -867,7 +867,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.1180059091711297</v>
+        <v>0.1235114882298213</v>
       </c>
     </row>
     <row r="45">
@@ -877,7 +877,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.1242790717772571</v>
+        <v>0.2225582301145566</v>
       </c>
     </row>
     <row r="46">
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.01759410569624674</v>
+        <v>0.109181001411259</v>
       </c>
     </row>
     <row r="47">
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.02247801664321289</v>
+        <v>0.09602225822789519</v>
       </c>
     </row>
     <row r="48">
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.02383726393173214</v>
+        <v>0.09318114877585877</v>
       </c>
     </row>
     <row r="49">
@@ -917,7 +917,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0.01615784618446613</v>
+        <v>0.1733513414591476</v>
       </c>
     </row>
     <row r="50">
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0.006770057605290907</v>
+        <v>0.1188506411471058</v>
       </c>
     </row>
     <row r="51">
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0.05552660545954176</v>
+        <v>0.09980937173357365</v>
       </c>
     </row>
     <row r="52">
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0.02314746135542888</v>
+        <v>0.09734677732880609</v>
       </c>
     </row>
     <row r="53">
@@ -957,7 +957,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.0460986752735657</v>
+        <v>0.1298539825571003</v>
       </c>
     </row>
     <row r="54">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>0.06999956736664419</v>
+        <v>0.1001172435372573</v>
       </c>
     </row>
     <row r="55">
@@ -977,7 +977,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0.06183401845617189</v>
+        <v>0.1390051992272035</v>
       </c>
     </row>
     <row r="56">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.005114075352960082</v>
+        <v>0.1258434492530135</v>
       </c>
     </row>
     <row r="57">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>0.07271078136469866</v>
+        <v>0.1167576391042217</v>
       </c>
     </row>
     <row r="58">
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>0</v>
+        <v>0.128041770789072</v>
       </c>
     </row>
     <row r="59">
@@ -1017,7 +1017,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>0.02730175511195892</v>
+        <v>0.0723155346026438</v>
       </c>
     </row>
     <row r="60">
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.03230332704781318</v>
+        <v>0.161634883982103</v>
       </c>
     </row>
     <row r="61">
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>0.01158219824001276</v>
+        <v>0.08852438687226048</v>
       </c>
     </row>
     <row r="62">
@@ -1047,7 +1047,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>0.06651010408592944</v>
+        <v>0.1213832020294272</v>
       </c>
     </row>
     <row r="63">
@@ -1057,7 +1057,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>0.06316767479480628</v>
+        <v>0.1083346132671438</v>
       </c>
     </row>
     <row r="64">
@@ -1067,7 +1067,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>0.05925013679933102</v>
+        <v>0.2085724839432637</v>
       </c>
     </row>
     <row r="65">
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.03039128874020515</v>
+        <v>0.1100033033587111</v>
       </c>
     </row>
     <row r="66">
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>0.06213455891740074</v>
+        <v>0.3416350265969719</v>
       </c>
     </row>
     <row r="67">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>0.03547782519733163</v>
+        <v>0.1119814139658299</v>
       </c>
     </row>
     <row r="68">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>0</v>
+        <v>0.07793712496896052</v>
       </c>
     </row>
     <row r="69">
@@ -1117,7 +1117,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>0.01422302934761605</v>
+        <v>0.105758376357277</v>
       </c>
     </row>
     <row r="70">
@@ -1127,7 +1127,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>0.0521319617915795</v>
+        <v>0.09561160183581252</v>
       </c>
     </row>
     <row r="71">
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0.003120045724398023</v>
+        <v>0.02123872576412017</v>
       </c>
     </row>
     <row r="72">
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>0.06040099052875397</v>
+        <v>0.09526936566216709</v>
       </c>
     </row>
     <row r="73">
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>0.07273213790251642</v>
+        <v>0.1492131184381201</v>
       </c>
     </row>
     <row r="74">
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>0.1592629973842256</v>
+        <v>0.194669989649316</v>
       </c>
     </row>
     <row r="75">
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>0.03912791663633923</v>
+        <v>0.06621449384672057</v>
       </c>
     </row>
     <row r="76">
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>0.2836089368663589</v>
+        <v>0.3340678059397715</v>
       </c>
     </row>
     <row r="77">
@@ -1197,7 +1197,7 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>0.02628458504708931</v>
+        <v>0.03736678270802618</v>
       </c>
     </row>
     <row r="78">
@@ -1207,7 +1207,7 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>0.05867721416740881</v>
+        <v>0.1175365968397262</v>
       </c>
     </row>
     <row r="79">
@@ -1217,7 +1217,7 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>0.1138570390388535</v>
+        <v>0.1441705428035616</v>
       </c>
     </row>
     <row r="80">
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>0.03280206956873437</v>
+        <v>0.09220062297247732</v>
       </c>
     </row>
     <row r="81">
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>0.06692387196920591</v>
+        <v>0.1434115754437097</v>
       </c>
     </row>
     <row r="82">
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>0.1611011254409812</v>
+        <v>0.1890083520746918</v>
       </c>
     </row>
     <row r="83">
@@ -1257,7 +1257,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0.02002505586033505</v>
+        <v>0.1144823272019987</v>
       </c>
     </row>
     <row r="84">
@@ -1267,7 +1267,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0.06219306383560161</v>
+        <v>0.1843926192449792</v>
       </c>
     </row>
     <row r="85">
@@ -1277,7 +1277,7 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>0.03391633620377789</v>
+        <v>0.1143485593388687</v>
       </c>
     </row>
     <row r="86">
@@ -1287,7 +1287,7 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0.1641822887326032</v>
+        <v>0.1700485803591078</v>
       </c>
     </row>
     <row r="87">
@@ -1297,7 +1297,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0.03984465070838782</v>
+        <v>0.08280420111691764</v>
       </c>
     </row>
     <row r="88">
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>0.01679716858469103</v>
+        <v>0.07253079122253671</v>
       </c>
     </row>
     <row r="89">
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>0.01470861350574691</v>
+        <v>0.1154726963119391</v>
       </c>
     </row>
     <row r="90">
@@ -1327,7 +1327,7 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>0.1403766086278063</v>
+        <v>0.2364207241836878</v>
       </c>
     </row>
     <row r="91">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>0.0579573685751102</v>
+        <v>0.218232762725021</v>
       </c>
     </row>
     <row r="92">
@@ -1347,7 +1347,7 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>0.01494364728414133</v>
+        <v>0.2332671059740414</v>
       </c>
     </row>
     <row r="93">
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>0.04261759458638211</v>
+        <v>0.09390443298818932</v>
       </c>
     </row>
     <row r="94">
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>0.07773356445574225</v>
+        <v>0.2812571459638914</v>
       </c>
     </row>
     <row r="95">
@@ -1377,7 +1377,7 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>0.08173030902532925</v>
+        <v>0.1103004129426448</v>
       </c>
     </row>
     <row r="96">
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>0.01915101375656999</v>
+        <v>0.047733910416302</v>
       </c>
     </row>
     <row r="97">
@@ -1397,7 +1397,7 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>0.05197872701274756</v>
+        <v>0.1584013268140441</v>
       </c>
     </row>
     <row r="98">
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>0.01144462086183384</v>
+        <v>0.05167696110255865</v>
       </c>
     </row>
     <row r="99">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>0.0773118363165028</v>
+        <v>0.1593869356239916</v>
       </c>
     </row>
     <row r="100">
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>0.0651714152359478</v>
+        <v>0.08544332018623031</v>
       </c>
     </row>
     <row r="101">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>0.07606329312440326</v>
+        <v>0.1143358073805528</v>
       </c>
     </row>
     <row r="102">
@@ -1447,7 +1447,7 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>0.002874903804186898</v>
+        <v>0.08137234975515326</v>
       </c>
     </row>
     <row r="103">
@@ -1457,7 +1457,7 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>0.07746812404201299</v>
+        <v>0.1658788515229492</v>
       </c>
     </row>
     <row r="104">
@@ -1467,7 +1467,7 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>0.02306644109730581</v>
+        <v>0.09849649761392962</v>
       </c>
     </row>
     <row r="105">
@@ -1477,7 +1477,7 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>0.06258726297918109</v>
+        <v>0.1888666780976486</v>
       </c>
     </row>
     <row r="106">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>0.01277780606931123</v>
+        <v>0.06817515658559439</v>
       </c>
     </row>
     <row r="107">
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>0.05564235268433307</v>
+        <v>0.1645533177736201</v>
       </c>
     </row>
     <row r="108">
@@ -1507,7 +1507,7 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>0.03701749369035906</v>
+        <v>0.08243982324399966</v>
       </c>
     </row>
     <row r="109">
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>0.08669382958594068</v>
+        <v>0.09330195892542148</v>
       </c>
     </row>
     <row r="110">
@@ -1527,7 +1527,7 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>0.02356741518494351</v>
+        <v>0.07643421723351229</v>
       </c>
     </row>
     <row r="111">
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>0.05881267475253225</v>
+        <v>0.1267908508278427</v>
       </c>
     </row>
     <row r="112">
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>0.01937681892961064</v>
+        <v>0.04037144199749194</v>
       </c>
     </row>
     <row r="113">
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>0.1040373421760337</v>
+        <v>0.1527709791505739</v>
       </c>
     </row>
     <row r="114">
@@ -1567,7 +1567,7 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>0.01160252211501756</v>
+        <v>0.03858989911269715</v>
       </c>
     </row>
     <row r="115">
@@ -1577,7 +1577,7 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>0.04749609488784992</v>
+        <v>0.2511839827711354</v>
       </c>
     </row>
     <row r="116">
@@ -1587,7 +1587,7 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>0.0119352124644408</v>
+        <v>0.03971831275740564</v>
       </c>
     </row>
     <row r="117">
@@ -1597,7 +1597,7 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>0.04286438374910398</v>
+        <v>0.106411630340976</v>
       </c>
     </row>
     <row r="118">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>0.05709698392735892</v>
+        <v>0.1147290864568175</v>
       </c>
     </row>
     <row r="119">
@@ -1617,7 +1617,7 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>0.02533831433060985</v>
+        <v>0.1368759892897662</v>
       </c>
     </row>
     <row r="120">
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>0.05334281544870161</v>
+        <v>0.0816732573777286</v>
       </c>
     </row>
     <row r="121">
@@ -1637,7 +1637,7 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>0.003068535390808119</v>
+        <v>0.1143900879132243</v>
       </c>
     </row>
     <row r="122">
@@ -1647,7 +1647,7 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>0.1055653955159132</v>
+        <v>0.210755343264642</v>
       </c>
     </row>
     <row r="123">
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="B123" t="n">
-        <v>0.01402495491831719</v>
+        <v>0.07692097654372856</v>
       </c>
     </row>
     <row r="124">
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="B124" t="n">
-        <v>0.08115695792166029</v>
+        <v>0.09607357259662884</v>
       </c>
     </row>
     <row r="125">
@@ -1677,7 +1677,7 @@
         </is>
       </c>
       <c r="B125" t="n">
-        <v>0.05153872424014368</v>
+        <v>0.2155755549065466</v>
       </c>
     </row>
     <row r="126">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="B126" t="n">
-        <v>0.0266948674104868</v>
+        <v>0.08306767717168538</v>
       </c>
     </row>
     <row r="127">
@@ -1697,7 +1697,7 @@
         </is>
       </c>
       <c r="B127" t="n">
-        <v>0.01759421713668659</v>
+        <v>0.04019266530671356</v>
       </c>
     </row>
     <row r="128">
@@ -1707,7 +1707,7 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>0.05904398860737576</v>
+        <v>0.1992220732516228</v>
       </c>
     </row>
     <row r="129">
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="B129" t="n">
-        <v>0.009009760102419606</v>
+        <v>0.1552558240972234</v>
       </c>
     </row>
     <row r="130">
@@ -1727,7 +1727,7 @@
         </is>
       </c>
       <c r="B130" t="n">
-        <v>0.064940325686778</v>
+        <v>0.07877542776947018</v>
       </c>
     </row>
     <row r="131">
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="B131" t="n">
-        <v>0.193362517029628</v>
+        <v>0.1940543046500162</v>
       </c>
     </row>
     <row r="132">
@@ -1747,7 +1747,7 @@
         </is>
       </c>
       <c r="B132" t="n">
-        <v>0.05829357035538173</v>
+        <v>0.1574819747169378</v>
       </c>
     </row>
     <row r="133">
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="B133" t="n">
-        <v>0.01036301495744246</v>
+        <v>0.121930493107522</v>
       </c>
     </row>
     <row r="134">
@@ -1767,7 +1767,7 @@
         </is>
       </c>
       <c r="B134" t="n">
-        <v>0.01631363033615486</v>
+        <v>0.08450247113041945</v>
       </c>
     </row>
     <row r="135">
@@ -1777,7 +1777,7 @@
         </is>
       </c>
       <c r="B135" t="n">
-        <v>0.001515461424993706</v>
+        <v>0.06475723794236568</v>
       </c>
     </row>
     <row r="136">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="B136" t="n">
-        <v>0.04282571331246435</v>
+        <v>0.1004429831514497</v>
       </c>
     </row>
     <row r="137">
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>0.005509093200907326</v>
+        <v>0.07165442375440503</v>
       </c>
     </row>
     <row r="138">
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="B138" t="n">
-        <v>0.01950404745071456</v>
+        <v>0.07329188201677402</v>
       </c>
     </row>
     <row r="139">
@@ -1817,7 +1817,7 @@
         </is>
       </c>
       <c r="B139" t="n">
-        <v>0.00527856754191606</v>
+        <v>0.125775496945088</v>
       </c>
     </row>
     <row r="140">
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="B140" t="n">
-        <v>0.04246568807000727</v>
+        <v>0.163005752279179</v>
       </c>
     </row>
     <row r="141">
@@ -1837,7 +1837,7 @@
         </is>
       </c>
       <c r="B141" t="n">
-        <v>0.05056742356168581</v>
+        <v>0.1554208178153123</v>
       </c>
     </row>
     <row r="142">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="B142" t="n">
-        <v>0.03920223562065663</v>
+        <v>0.09409797753071605</v>
       </c>
     </row>
     <row r="143">
@@ -1857,7 +1857,7 @@
         </is>
       </c>
       <c r="B143" t="n">
-        <v>0.02436009630091038</v>
+        <v>0.08111802495264701</v>
       </c>
     </row>
     <row r="144">
@@ -1867,7 +1867,7 @@
         </is>
       </c>
       <c r="B144" t="n">
-        <v>0.002140304838763128</v>
+        <v>0.05822734078971207</v>
       </c>
     </row>
     <row r="145">
@@ -1877,7 +1877,7 @@
         </is>
       </c>
       <c r="B145" t="n">
-        <v>0.04871529731043408</v>
+        <v>0.09499355531983072</v>
       </c>
     </row>
     <row r="146">
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="B146" t="n">
-        <v>0.02923530729557648</v>
+        <v>0.1251696834079427</v>
       </c>
     </row>
     <row r="147">
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="B147" t="n">
-        <v>0.07966276035567001</v>
+        <v>0.1353107959274259</v>
       </c>
     </row>
     <row r="148">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="B148" t="n">
-        <v>0.01254373252347789</v>
+        <v>0.1487886950121503</v>
       </c>
     </row>
     <row r="149">
@@ -1917,7 +1917,7 @@
         </is>
       </c>
       <c r="B149" t="n">
-        <v>0.005206736090263518</v>
+        <v>0.02517786200895248</v>
       </c>
     </row>
     <row r="150">
@@ -1927,7 +1927,7 @@
         </is>
       </c>
       <c r="B150" t="n">
-        <v>0.04899765562457404</v>
+        <v>0.1146451682554864</v>
       </c>
     </row>
     <row r="151">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="B151" t="n">
-        <v>0.04190999997143956</v>
+        <v>0.0669626008348215</v>
       </c>
     </row>
     <row r="152">
@@ -1947,7 +1947,7 @@
         </is>
       </c>
       <c r="B152" t="n">
-        <v>0.1365830098518232</v>
+        <v>0.1768266608237921</v>
       </c>
     </row>
     <row r="153">
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="B153" t="n">
-        <v>0.01851769155365434</v>
+        <v>0.05653180278820311</v>
       </c>
     </row>
     <row r="154">
@@ -1967,7 +1967,7 @@
         </is>
       </c>
       <c r="B154" t="n">
-        <v>0.04887513750650058</v>
+        <v>0.1094841892636169</v>
       </c>
     </row>
     <row r="155">
@@ -1977,7 +1977,7 @@
         </is>
       </c>
       <c r="B155" t="n">
-        <v>0.01064429775082058</v>
+        <v>0.03773464935423581</v>
       </c>
     </row>
     <row r="156">
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="B156" t="n">
-        <v>0.04273658551000159</v>
+        <v>0.0981101307883315</v>
       </c>
     </row>
     <row r="157">
@@ -1997,7 +1997,7 @@
         </is>
       </c>
       <c r="B157" t="n">
-        <v>0.09081534743376399</v>
+        <v>0.1254497091859273</v>
       </c>
     </row>
     <row r="158">
@@ -2007,7 +2007,7 @@
         </is>
       </c>
       <c r="B158" t="n">
-        <v>0.01321265134044672</v>
+        <v>0.2306655944625516</v>
       </c>
     </row>
     <row r="159">
@@ -2017,7 +2017,7 @@
         </is>
       </c>
       <c r="B159" t="n">
-        <v>0.03826023828273568</v>
+        <v>0.1001656676283235</v>
       </c>
     </row>
     <row r="160">
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="B160" t="n">
-        <v>0.06617763929013189</v>
+        <v>0.1299082357254308</v>
       </c>
     </row>
     <row r="161">
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="B161" t="n">
-        <v>0.0506635854947652</v>
+        <v>0.06806465643172528</v>
       </c>
     </row>
     <row r="162">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="B162" t="n">
-        <v>0.04812852239575097</v>
+        <v>0.09868528241640426</v>
       </c>
     </row>
     <row r="163">
@@ -2057,7 +2057,7 @@
         </is>
       </c>
       <c r="B163" t="n">
-        <v>0.03909630874271292</v>
+        <v>0.1359294544585445</v>
       </c>
     </row>
     <row r="164">
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="B164" t="n">
-        <v>0.03319418895261873</v>
+        <v>0.1127041822447714</v>
       </c>
     </row>
     <row r="165">
@@ -2077,7 +2077,7 @@
         </is>
       </c>
       <c r="B165" t="n">
-        <v>0.04407485556323599</v>
+        <v>0.108692474075889</v>
       </c>
     </row>
     <row r="166">
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="B166" t="n">
-        <v>0.03327985389059664</v>
+        <v>0.03910188801541346</v>
       </c>
     </row>
     <row r="167">
@@ -2097,7 +2097,7 @@
         </is>
       </c>
       <c r="B167" t="n">
-        <v>0.08202239906555132</v>
+        <v>0.1337004881628295</v>
       </c>
     </row>
     <row r="168">
@@ -2107,7 +2107,7 @@
         </is>
       </c>
       <c r="B168" t="n">
-        <v>0.06513315619484453</v>
+        <v>0.1700276618319278</v>
       </c>
     </row>
     <row r="169">
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="B169" t="n">
-        <v>0.02594000156084749</v>
+        <v>0.05170547584788417</v>
       </c>
     </row>
     <row r="170">
@@ -2127,7 +2127,7 @@
         </is>
       </c>
       <c r="B170" t="n">
-        <v>0.000127097674983443</v>
+        <v>0.01707145585074406</v>
       </c>
     </row>
     <row r="171">
@@ -2137,7 +2137,7 @@
         </is>
       </c>
       <c r="B171" t="n">
-        <v>0.02929478372420099</v>
+        <v>0.1107495298418665</v>
       </c>
     </row>
     <row r="172">
@@ -2147,7 +2147,7 @@
         </is>
       </c>
       <c r="B172" t="n">
-        <v>0.03297754521894145</v>
+        <v>0.0593540248032399</v>
       </c>
     </row>
     <row r="173">
@@ -2157,7 +2157,7 @@
         </is>
       </c>
       <c r="B173" t="n">
-        <v>0.04324794548517514</v>
+        <v>0.1422925918130153</v>
       </c>
     </row>
     <row r="174">
@@ -2167,7 +2167,7 @@
         </is>
       </c>
       <c r="B174" t="n">
-        <v>0.09261996291704036</v>
+        <v>0.1424447864329434</v>
       </c>
     </row>
     <row r="175">
@@ -2177,7 +2177,7 @@
         </is>
       </c>
       <c r="B175" t="n">
-        <v>0.02285092104661254</v>
+        <v>0.1473087643808161</v>
       </c>
     </row>
     <row r="176">
@@ -2187,7 +2187,7 @@
         </is>
       </c>
       <c r="B176" t="n">
-        <v>0.01776999811830111</v>
+        <v>0.07157598117396174</v>
       </c>
     </row>
     <row r="177">
@@ -2197,7 +2197,7 @@
         </is>
       </c>
       <c r="B177" t="n">
-        <v>0.008080916005068281</v>
+        <v>0.1289435172471209</v>
       </c>
     </row>
     <row r="178">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="B178" t="n">
-        <v>0.02772429726607624</v>
+        <v>0.04892101426669559</v>
       </c>
     </row>
     <row r="179">
@@ -2217,7 +2217,7 @@
         </is>
       </c>
       <c r="B179" t="n">
-        <v>0</v>
+        <v>0.1161940737123843</v>
       </c>
     </row>
     <row r="180">
@@ -2227,7 +2227,7 @@
         </is>
       </c>
       <c r="B180" t="n">
-        <v>0.05023237538109274</v>
+        <v>0.2218036969784996</v>
       </c>
     </row>
     <row r="181">
@@ -2237,7 +2237,7 @@
         </is>
       </c>
       <c r="B181" t="n">
-        <v>0.1266013186850364</v>
+        <v>0.1404050070712477</v>
       </c>
     </row>
     <row r="182">
@@ -2247,7 +2247,7 @@
         </is>
       </c>
       <c r="B182" t="n">
-        <v>0.1014393864394245</v>
+        <v>0.171189640080603</v>
       </c>
     </row>
     <row r="183">
@@ -2257,7 +2257,7 @@
         </is>
       </c>
       <c r="B183" t="n">
-        <v>0.148428346473611</v>
+        <v>0.1939417141692804</v>
       </c>
     </row>
     <row r="184">
@@ -2267,7 +2267,7 @@
         </is>
       </c>
       <c r="B184" t="n">
-        <v>0.08612670327591757</v>
+        <v>0.1985705863293632</v>
       </c>
     </row>
     <row r="185">
@@ -2277,7 +2277,7 @@
         </is>
       </c>
       <c r="B185" t="n">
-        <v>0.02094173175487246</v>
+        <v>0.1797430857202199</v>
       </c>
     </row>
     <row r="186">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="B186" t="n">
-        <v>0.002101852624900667</v>
+        <v>0.02664524213141246</v>
       </c>
     </row>
     <row r="187">
@@ -2297,7 +2297,7 @@
         </is>
       </c>
       <c r="B187" t="n">
-        <v>0.001730606490250652</v>
+        <v>0.1029542746282602</v>
       </c>
     </row>
     <row r="188">
@@ -2307,7 +2307,7 @@
         </is>
       </c>
       <c r="B188" t="n">
-        <v>0.2395509556592278</v>
+        <v>0.2659657749837693</v>
       </c>
     </row>
     <row r="189">
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="B189" t="n">
-        <v>0.08433607596627511</v>
+        <v>0.126643622691735</v>
       </c>
     </row>
     <row r="190">
@@ -2327,7 +2327,7 @@
         </is>
       </c>
       <c r="B190" t="n">
-        <v>0.02872786939817806</v>
+        <v>0.07373243314306047</v>
       </c>
     </row>
     <row r="191">
@@ -2337,7 +2337,7 @@
         </is>
       </c>
       <c r="B191" t="n">
-        <v>0.005749402309907535</v>
+        <v>0.06222755008344902</v>
       </c>
     </row>
     <row r="192">
@@ -2347,7 +2347,7 @@
         </is>
       </c>
       <c r="B192" t="n">
-        <v>0.03885758476669594</v>
+        <v>0.09576781210260379</v>
       </c>
     </row>
     <row r="193">
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c r="B193" t="n">
-        <v>0.08313544992123775</v>
+        <v>0.1965801264269451</v>
       </c>
     </row>
     <row r="194">
@@ -2367,7 +2367,7 @@
         </is>
       </c>
       <c r="B194" t="n">
-        <v>0.01286543763916403</v>
+        <v>0.1326254432213582</v>
       </c>
     </row>
     <row r="195">
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="B195" t="n">
-        <v>0.03922753619853601</v>
+        <v>0.1116756161221629</v>
       </c>
     </row>
     <row r="196">
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="B196" t="n">
-        <v>0.04635937575391105</v>
+        <v>0.08533964212384859</v>
       </c>
     </row>
     <row r="197">
@@ -2397,7 +2397,7 @@
         </is>
       </c>
       <c r="B197" t="n">
-        <v>0.01387920768048898</v>
+        <v>0.1365537046958244</v>
       </c>
     </row>
     <row r="198">
@@ -2407,7 +2407,7 @@
         </is>
       </c>
       <c r="B198" t="n">
-        <v>0.04420256709193038</v>
+        <v>0.09909266208868008</v>
       </c>
     </row>
     <row r="199">
@@ -2417,7 +2417,7 @@
         </is>
       </c>
       <c r="B199" t="n">
-        <v>0.02592697097384833</v>
+        <v>0.265243341793564</v>
       </c>
     </row>
     <row r="200">
@@ -2427,7 +2427,7 @@
         </is>
       </c>
       <c r="B200" t="n">
-        <v>0.02823760589878503</v>
+        <v>0.05682783235328698</v>
       </c>
     </row>
     <row r="201">
@@ -2437,7 +2437,7 @@
         </is>
       </c>
       <c r="B201" t="n">
-        <v>0.05390095215282231</v>
+        <v>0.2070384894434664</v>
       </c>
     </row>
     <row r="202">
@@ -2447,7 +2447,7 @@
         </is>
       </c>
       <c r="B202" t="n">
-        <v>0.01869446959848284</v>
+        <v>0.09981198388878783</v>
       </c>
     </row>
     <row r="203">
@@ -2457,7 +2457,7 @@
         </is>
       </c>
       <c r="B203" t="n">
-        <v>0.07291741117682084</v>
+        <v>0.1318715729887368</v>
       </c>
     </row>
     <row r="204">
@@ -2467,7 +2467,7 @@
         </is>
       </c>
       <c r="B204" t="n">
-        <v>0.02457196349998823</v>
+        <v>0.1303339695747832</v>
       </c>
     </row>
     <row r="205">
@@ -2477,7 +2477,7 @@
         </is>
       </c>
       <c r="B205" t="n">
-        <v>0.001223901835394966</v>
+        <v>0.05970941926046534</v>
       </c>
     </row>
     <row r="206">
@@ -2487,7 +2487,7 @@
         </is>
       </c>
       <c r="B206" t="n">
-        <v>0.02244177977418839</v>
+        <v>0.07036319546528401</v>
       </c>
     </row>
     <row r="207">
@@ -2497,7 +2497,7 @@
         </is>
       </c>
       <c r="B207" t="n">
-        <v>0</v>
+        <v>0.2171769079056559</v>
       </c>
     </row>
     <row r="208">
@@ -2507,7 +2507,7 @@
         </is>
       </c>
       <c r="B208" t="n">
-        <v>0.05697194731350635</v>
+        <v>0.1713874532206945</v>
       </c>
     </row>
     <row r="209">
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="B209" t="n">
-        <v>0.03339555134815245</v>
+        <v>0.1227747200218288</v>
       </c>
     </row>
     <row r="210">
@@ -2527,7 +2527,7 @@
         </is>
       </c>
       <c r="B210" t="n">
-        <v>0.07490400346564009</v>
+        <v>0.1510908570151192</v>
       </c>
     </row>
     <row r="211">
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="B211" t="n">
-        <v>0.04540657463208835</v>
+        <v>0.08468105803504783</v>
       </c>
     </row>
     <row r="212">
@@ -2547,7 +2547,7 @@
         </is>
       </c>
       <c r="B212" t="n">
-        <v>0.02833030274487904</v>
+        <v>0.1216089966008261</v>
       </c>
     </row>
     <row r="213">
@@ -2557,7 +2557,7 @@
         </is>
       </c>
       <c r="B213" t="n">
-        <v>0.001874753931355164</v>
+        <v>0.0364799033750809</v>
       </c>
     </row>
     <row r="214">
@@ -2567,7 +2567,7 @@
         </is>
       </c>
       <c r="B214" t="n">
-        <v>0.0493983356617153</v>
+        <v>0.180201386481143</v>
       </c>
     </row>
     <row r="215">
@@ -2577,7 +2577,7 @@
         </is>
       </c>
       <c r="B215" t="n">
-        <v>0.04902956176127102</v>
+        <v>0.137400283825863</v>
       </c>
     </row>
     <row r="216">
@@ -2587,7 +2587,7 @@
         </is>
       </c>
       <c r="B216" t="n">
-        <v>0.03712235766793482</v>
+        <v>0.1720225602287922</v>
       </c>
     </row>
     <row r="217">
@@ -2597,7 +2597,7 @@
         </is>
       </c>
       <c r="B217" t="n">
-        <v>0.03487312871824241</v>
+        <v>0.1491111387323941</v>
       </c>
     </row>
     <row r="218">
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="B218" t="n">
-        <v>0.10730388541309</v>
+        <v>0.1313954518811227</v>
       </c>
     </row>
     <row r="219">
@@ -2617,7 +2617,7 @@
         </is>
       </c>
       <c r="B219" t="n">
-        <v>0.02327872693452672</v>
+        <v>0.04359209844936369</v>
       </c>
     </row>
     <row r="220">
@@ -2627,7 +2627,7 @@
         </is>
       </c>
       <c r="B220" t="n">
-        <v>0.03305342083806343</v>
+        <v>0.1505830522611281</v>
       </c>
     </row>
     <row r="221">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="B221" t="n">
-        <v>0.01351990399217247</v>
+        <v>0.06586012432811794</v>
       </c>
     </row>
     <row r="222">
@@ -2647,7 +2647,7 @@
         </is>
       </c>
       <c r="B222" t="n">
-        <v>0.1021119056504051</v>
+        <v>0.1667482264782105</v>
       </c>
     </row>
     <row r="223">
@@ -2657,7 +2657,7 @@
         </is>
       </c>
       <c r="B223" t="n">
-        <v>0.09541244164900053</v>
+        <v>0.1994501193600927</v>
       </c>
     </row>
     <row r="224">
@@ -2667,7 +2667,7 @@
         </is>
       </c>
       <c r="B224" t="n">
-        <v>0.04203626556563723</v>
+        <v>0.1028639268094186</v>
       </c>
     </row>
     <row r="225">
@@ -2677,7 +2677,7 @@
         </is>
       </c>
       <c r="B225" t="n">
-        <v>0.04312017116144776</v>
+        <v>0.1869002982687857</v>
       </c>
     </row>
     <row r="226">
@@ -2687,7 +2687,7 @@
         </is>
       </c>
       <c r="B226" t="n">
-        <v>0.04949722449469105</v>
+        <v>0.1884122523177946</v>
       </c>
     </row>
     <row r="227">
@@ -2697,7 +2697,7 @@
         </is>
       </c>
       <c r="B227" t="n">
-        <v>0.0510365652858142</v>
+        <v>0.06427077581994273</v>
       </c>
     </row>
     <row r="228">
@@ -2707,7 +2707,7 @@
         </is>
       </c>
       <c r="B228" t="n">
-        <v>0.01916788769148348</v>
+        <v>0.06351759775665827</v>
       </c>
     </row>
     <row r="229">
@@ -2717,7 +2717,7 @@
         </is>
       </c>
       <c r="B229" t="n">
-        <v>0.02262150612944771</v>
+        <v>0.03492967746700531</v>
       </c>
     </row>
     <row r="230">
@@ -2727,7 +2727,7 @@
         </is>
       </c>
       <c r="B230" t="n">
-        <v>0.03563075157194334</v>
+        <v>0.0731326261832617</v>
       </c>
     </row>
     <row r="231">
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="B231" t="n">
-        <v>0.03512398945120746</v>
+        <v>0.1952538727994642</v>
       </c>
     </row>
     <row r="232">
@@ -2747,7 +2747,7 @@
         </is>
       </c>
       <c r="B232" t="n">
-        <v>0.08903984593906239</v>
+        <v>0.1853286896377574</v>
       </c>
     </row>
     <row r="233">
@@ -2757,7 +2757,7 @@
         </is>
       </c>
       <c r="B233" t="n">
-        <v>0.004255740212859209</v>
+        <v>0.05361452884066909</v>
       </c>
     </row>
     <row r="234">
@@ -2767,7 +2767,7 @@
         </is>
       </c>
       <c r="B234" t="n">
-        <v>0.0609511341076723</v>
+        <v>0.1003387661992871</v>
       </c>
     </row>
     <row r="235">
@@ -2777,7 +2777,7 @@
         </is>
       </c>
       <c r="B235" t="n">
-        <v>0.02480153468881599</v>
+        <v>0.1553006646334633</v>
       </c>
     </row>
     <row r="236">
@@ -2787,7 +2787,7 @@
         </is>
       </c>
       <c r="B236" t="n">
-        <v>0.02502767799229672</v>
+        <v>0.08658085632632738</v>
       </c>
     </row>
     <row r="237">
@@ -2797,7 +2797,7 @@
         </is>
       </c>
       <c r="B237" t="n">
-        <v>0.117374387050641</v>
+        <v>0.1666747679819775</v>
       </c>
     </row>
     <row r="238">
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="B238" t="n">
-        <v>0.08640629938464918</v>
+        <v>0.150268663027158</v>
       </c>
     </row>
     <row r="239">
@@ -2817,7 +2817,7 @@
         </is>
       </c>
       <c r="B239" t="n">
-        <v>0.03328741834224124</v>
+        <v>0.1192989920775588</v>
       </c>
     </row>
     <row r="240">
@@ -2827,7 +2827,7 @@
         </is>
       </c>
       <c r="B240" t="n">
-        <v>0.02525229205457617</v>
+        <v>0.09525962153412142</v>
       </c>
     </row>
     <row r="241">
@@ -2837,7 +2837,7 @@
         </is>
       </c>
       <c r="B241" t="n">
-        <v>0.06612176807028322</v>
+        <v>0.09443450131620174</v>
       </c>
     </row>
     <row r="242">
@@ -2847,7 +2847,7 @@
         </is>
       </c>
       <c r="B242" t="n">
-        <v>0.05197817238907173</v>
+        <v>0.1641256793023157</v>
       </c>
     </row>
     <row r="243">
@@ -2857,7 +2857,7 @@
         </is>
       </c>
       <c r="B243" t="n">
-        <v>0.008191722625582322</v>
+        <v>0.1533889365414797</v>
       </c>
     </row>
     <row r="244">
@@ -2867,7 +2867,7 @@
         </is>
       </c>
       <c r="B244" t="n">
-        <v>0.02954223361634641</v>
+        <v>0.09876295097440521</v>
       </c>
     </row>
     <row r="245">
@@ -2877,7 +2877,7 @@
         </is>
       </c>
       <c r="B245" t="n">
-        <v>0.06679864755206778</v>
+        <v>0.1356429415697624</v>
       </c>
     </row>
     <row r="246">
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="B246" t="n">
-        <v>0.0708332297582881</v>
+        <v>0.1440937963102781</v>
       </c>
     </row>
     <row r="247">
@@ -2897,7 +2897,7 @@
         </is>
       </c>
       <c r="B247" t="n">
-        <v>0.04661031365601685</v>
+        <v>0.115521744343505</v>
       </c>
     </row>
     <row r="248">
@@ -2907,7 +2907,7 @@
         </is>
       </c>
       <c r="B248" t="n">
-        <v>0.0723153770731525</v>
+        <v>0.1752242291410064</v>
       </c>
     </row>
     <row r="249">
@@ -2917,7 +2917,7 @@
         </is>
       </c>
       <c r="B249" t="n">
-        <v>0.0605107157129359</v>
+        <v>0.1071121269395942</v>
       </c>
     </row>
     <row r="250">
@@ -2927,7 +2927,7 @@
         </is>
       </c>
       <c r="B250" t="n">
-        <v>0.1389352554740336</v>
+        <v>0.2301576063805217</v>
       </c>
     </row>
     <row r="251">
@@ -2937,7 +2937,7 @@
         </is>
       </c>
       <c r="B251" t="n">
-        <v>0.06347676385111696</v>
+        <v>0.2557378479392075</v>
       </c>
     </row>
     <row r="252">
@@ -2947,7 +2947,7 @@
         </is>
       </c>
       <c r="B252" t="n">
-        <v>0.07970736482978004</v>
+        <v>0.1115650664338738</v>
       </c>
     </row>
     <row r="253">
@@ -2957,7 +2957,7 @@
         </is>
       </c>
       <c r="B253" t="n">
-        <v>0.03983388607971956</v>
+        <v>0.1059950926993541</v>
       </c>
     </row>
     <row r="254">
@@ -2967,7 +2967,7 @@
         </is>
       </c>
       <c r="B254" t="n">
-        <v>0.03185363920680049</v>
+        <v>0.1047469432948983</v>
       </c>
     </row>
     <row r="255">
@@ -2977,7 +2977,7 @@
         </is>
       </c>
       <c r="B255" t="n">
-        <v>0.01304958982206243</v>
+        <v>0.04675246613888298</v>
       </c>
     </row>
     <row r="256">
@@ -2987,7 +2987,7 @@
         </is>
       </c>
       <c r="B256" t="n">
-        <v>0.2349627788858671</v>
+        <v>0.3020635715992724</v>
       </c>
     </row>
     <row r="257">
@@ -2997,7 +2997,7 @@
         </is>
       </c>
       <c r="B257" t="n">
-        <v>0.078240708003736</v>
+        <v>0.1173620111052226</v>
       </c>
     </row>
     <row r="258">
@@ -3007,7 +3007,7 @@
         </is>
       </c>
       <c r="B258" t="n">
-        <v>0.002524908841057994</v>
+        <v>0.09743058062108466</v>
       </c>
     </row>
     <row r="259">
@@ -3017,7 +3017,7 @@
         </is>
       </c>
       <c r="B259" t="n">
-        <v>0.02849391212541904</v>
+        <v>0.06332547048446099</v>
       </c>
     </row>
     <row r="260">
@@ -3027,7 +3027,7 @@
         </is>
       </c>
       <c r="B260" t="n">
-        <v>0.06103389343242571</v>
+        <v>0.08823793962484774</v>
       </c>
     </row>
     <row r="261">
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="B261" t="n">
-        <v>0</v>
+        <v>0.2475316306988126</v>
       </c>
     </row>
     <row r="262">
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="B262" t="n">
-        <v>0.02366410110442927</v>
+        <v>0.07598157770781609</v>
       </c>
     </row>
     <row r="263">
@@ -3057,7 +3057,7 @@
         </is>
       </c>
       <c r="B263" t="n">
-        <v>0.01000049861138433</v>
+        <v>0.03160571583416116</v>
       </c>
     </row>
     <row r="264">
@@ -3067,7 +3067,7 @@
         </is>
       </c>
       <c r="B264" t="n">
-        <v>0.05236924977007811</v>
+        <v>0.1372845619390566</v>
       </c>
     </row>
     <row r="265">
@@ -3077,7 +3077,7 @@
         </is>
       </c>
       <c r="B265" t="n">
-        <v>0.1649638807494482</v>
+        <v>0.1995441470001623</v>
       </c>
     </row>
     <row r="266">
@@ -3087,7 +3087,7 @@
         </is>
       </c>
       <c r="B266" t="n">
-        <v>0.01504615548551557</v>
+        <v>0.08231873419250578</v>
       </c>
     </row>
     <row r="267">
@@ -3097,7 +3097,7 @@
         </is>
       </c>
       <c r="B267" t="n">
-        <v>0.0120940250873706</v>
+        <v>0.05789647487584666</v>
       </c>
     </row>
     <row r="268">
@@ -3107,7 +3107,7 @@
         </is>
       </c>
       <c r="B268" t="n">
-        <v>0.00117024875995026</v>
+        <v>0.05393603056041228</v>
       </c>
     </row>
     <row r="269">
@@ -3117,7 +3117,7 @@
         </is>
       </c>
       <c r="B269" t="n">
-        <v>0.1228611762160168</v>
+        <v>0.1792428753802993</v>
       </c>
     </row>
     <row r="270">
@@ -3127,7 +3127,7 @@
         </is>
       </c>
       <c r="B270" t="n">
-        <v>0.1703983613504732</v>
+        <v>0.2378541093516024</v>
       </c>
     </row>
     <row r="271">
@@ -3137,7 +3137,7 @@
         </is>
       </c>
       <c r="B271" t="n">
-        <v>0.0943428421309959</v>
+        <v>0.1377083619636598</v>
       </c>
     </row>
     <row r="272">
@@ -3147,7 +3147,7 @@
         </is>
       </c>
       <c r="B272" t="n">
-        <v>0.01895179081925137</v>
+        <v>0.1282246487450222</v>
       </c>
     </row>
     <row r="273">
@@ -3157,7 +3157,7 @@
         </is>
       </c>
       <c r="B273" t="n">
-        <v>0.03619689805278629</v>
+        <v>0.1379635218286192</v>
       </c>
     </row>
     <row r="274">
@@ -3167,7 +3167,7 @@
         </is>
       </c>
       <c r="B274" t="n">
-        <v>0.01147743843727363</v>
+        <v>0.15000244590896</v>
       </c>
     </row>
     <row r="275">
@@ -3177,7 +3177,7 @@
         </is>
       </c>
       <c r="B275" t="n">
-        <v>0.07442567860624955</v>
+        <v>0.09122254515877795</v>
       </c>
     </row>
     <row r="276">
@@ -3187,7 +3187,7 @@
         </is>
       </c>
       <c r="B276" t="n">
-        <v>0.01050557305630072</v>
+        <v>0.05856134667689549</v>
       </c>
     </row>
     <row r="277">
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="B277" t="n">
-        <v>0.005977873550820502</v>
+        <v>0.03993043682501986</v>
       </c>
     </row>
     <row r="278">
@@ -3207,7 +3207,7 @@
         </is>
       </c>
       <c r="B278" t="n">
-        <v>0.02113069116950765</v>
+        <v>0.1264584795671897</v>
       </c>
     </row>
     <row r="279">
@@ -3217,7 +3217,7 @@
         </is>
       </c>
       <c r="B279" t="n">
-        <v>0.04400709468640886</v>
+        <v>0.1185418384847713</v>
       </c>
     </row>
     <row r="280">
@@ -3227,7 +3227,7 @@
         </is>
       </c>
       <c r="B280" t="n">
-        <v>0.01918404584213141</v>
+        <v>0.04964600410062615</v>
       </c>
     </row>
     <row r="281">
@@ -3237,7 +3237,7 @@
         </is>
       </c>
       <c r="B281" t="n">
-        <v>0</v>
+        <v>0.258906536048065</v>
       </c>
     </row>
     <row r="282">
@@ -3247,7 +3247,7 @@
         </is>
       </c>
       <c r="B282" t="n">
-        <v>0</v>
+        <v>0.03634956338755424</v>
       </c>
     </row>
     <row r="283">
@@ -3257,7 +3257,7 @@
         </is>
       </c>
       <c r="B283" t="n">
-        <v>0.001234688464506173</v>
+        <v>0.05885242518960308</v>
       </c>
     </row>
     <row r="284">
@@ -3267,7 +3267,7 @@
         </is>
       </c>
       <c r="B284" t="n">
-        <v>0.02534854265330474</v>
+        <v>0.08061408518844067</v>
       </c>
     </row>
     <row r="285">
@@ -3277,7 +3277,7 @@
         </is>
       </c>
       <c r="B285" t="n">
-        <v>0.02997245179063361</v>
+        <v>0.1755447083183012</v>
       </c>
     </row>
     <row r="286">
@@ -3287,7 +3287,7 @@
         </is>
       </c>
       <c r="B286" t="n">
-        <v>0.001121273742086586</v>
+        <v>0.0191902041220318</v>
       </c>
     </row>
     <row r="287">
@@ -3297,7 +3297,7 @@
         </is>
       </c>
       <c r="B287" t="n">
-        <v>0.02834754599684087</v>
+        <v>0.07273753231649864</v>
       </c>
     </row>
     <row r="288">
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="B288" t="n">
-        <v>0.110691200261492</v>
+        <v>0.1483531284274327</v>
       </c>
     </row>
     <row r="289">
@@ -3317,7 +3317,7 @@
         </is>
       </c>
       <c r="B289" t="n">
-        <v>0.07751364232715698</v>
+        <v>0.1410400651054648</v>
       </c>
     </row>
     <row r="290">
@@ -3327,7 +3327,7 @@
         </is>
       </c>
       <c r="B290" t="n">
-        <v>0.1298813082418485</v>
+        <v>0.1994403301843231</v>
       </c>
     </row>
     <row r="291">
@@ -3337,7 +3337,7 @@
         </is>
       </c>
       <c r="B291" t="n">
-        <v>0.009275633999733615</v>
+        <v>0.05409827725135337</v>
       </c>
     </row>
     <row r="292">
@@ -3347,7 +3347,7 @@
         </is>
       </c>
       <c r="B292" t="n">
-        <v>0.01114768479706786</v>
+        <v>0.08927767045660506</v>
       </c>
     </row>
     <row r="293">
@@ -3357,7 +3357,7 @@
         </is>
       </c>
       <c r="B293" t="n">
-        <v>0.06879347721224269</v>
+        <v>0.1027087752716248</v>
       </c>
     </row>
     <row r="294">
@@ -3367,7 +3367,7 @@
         </is>
       </c>
       <c r="B294" t="n">
-        <v>0.05208210514381306</v>
+        <v>0.1941526176133529</v>
       </c>
     </row>
     <row r="295">
@@ -3377,7 +3377,7 @@
         </is>
       </c>
       <c r="B295" t="n">
-        <v>0</v>
+        <v>0.05384789141321341</v>
       </c>
     </row>
     <row r="296">
@@ -3387,7 +3387,7 @@
         </is>
       </c>
       <c r="B296" t="n">
-        <v>0.02497671156977996</v>
+        <v>0.04527993542861183</v>
       </c>
     </row>
     <row r="297">
@@ -3397,7 +3397,7 @@
         </is>
       </c>
       <c r="B297" t="n">
-        <v>0.00662374734578946</v>
+        <v>0.1104125035808724</v>
       </c>
     </row>
     <row r="298">
@@ -3407,7 +3407,7 @@
         </is>
       </c>
       <c r="B298" t="n">
-        <v>0.04155087524891863</v>
+        <v>0.1222314171051482</v>
       </c>
     </row>
     <row r="299">
@@ -3417,7 +3417,7 @@
         </is>
       </c>
       <c r="B299" t="n">
-        <v>0.03927233695633622</v>
+        <v>0.140317836497761</v>
       </c>
     </row>
     <row r="300">
@@ -3427,7 +3427,7 @@
         </is>
       </c>
       <c r="B300" t="n">
-        <v>0.02674929805475001</v>
+        <v>0.1436243286094551</v>
       </c>
     </row>
     <row r="301">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="B301" t="n">
-        <v>0.05414704213581011</v>
+        <v>0.266645807413994</v>
       </c>
     </row>
     <row r="302">
@@ -3447,7 +3447,7 @@
         </is>
       </c>
       <c r="B302" t="n">
-        <v>0.03270561482269627</v>
+        <v>0.1112655096155932</v>
       </c>
     </row>
     <row r="303">
@@ -3457,7 +3457,7 @@
         </is>
       </c>
       <c r="B303" t="n">
-        <v>0.01645629419455836</v>
+        <v>0.04754922220382366</v>
       </c>
     </row>
     <row r="304">
@@ -3467,7 +3467,7 @@
         </is>
       </c>
       <c r="B304" t="n">
-        <v>0</v>
+        <v>0.008679133298288984</v>
       </c>
     </row>
     <row r="305">
@@ -3477,7 +3477,7 @@
         </is>
       </c>
       <c r="B305" t="n">
-        <v>0.07202012025369933</v>
+        <v>0.1354218884582049</v>
       </c>
     </row>
     <row r="306">
@@ -3487,7 +3487,7 @@
         </is>
       </c>
       <c r="B306" t="n">
-        <v>0</v>
+        <v>0.143460120388141</v>
       </c>
     </row>
     <row r="307">
@@ -3497,7 +3497,7 @@
         </is>
       </c>
       <c r="B307" t="n">
-        <v>0.02003409472976848</v>
+        <v>0.06937642651792338</v>
       </c>
     </row>
     <row r="308">
@@ -3507,7 +3507,7 @@
         </is>
       </c>
       <c r="B308" t="n">
-        <v>0.01615278271895926</v>
+        <v>0.04463350319393799</v>
       </c>
     </row>
     <row r="309">
@@ -3517,7 +3517,7 @@
         </is>
       </c>
       <c r="B309" t="n">
-        <v>0.01699399488760691</v>
+        <v>0.1663666460177142</v>
       </c>
     </row>
     <row r="310">
@@ -3527,7 +3527,7 @@
         </is>
       </c>
       <c r="B310" t="n">
-        <v>0.1157057861923274</v>
+        <v>0.1150732818545804</v>
       </c>
     </row>
     <row r="311">
@@ -3537,7 +3537,7 @@
         </is>
       </c>
       <c r="B311" t="n">
-        <v>0.01506176167940557</v>
+        <v>0.119932601351483</v>
       </c>
     </row>
     <row r="312">
@@ -3547,7 +3547,7 @@
         </is>
       </c>
       <c r="B312" t="n">
-        <v>0</v>
+        <v>0.05989417516840648</v>
       </c>
     </row>
     <row r="313">
@@ -3557,7 +3557,7 @@
         </is>
       </c>
       <c r="B313" t="n">
-        <v>0.1260329671690593</v>
+        <v>0.2801325381460434</v>
       </c>
     </row>
     <row r="314">
@@ -3567,7 +3567,7 @@
         </is>
       </c>
       <c r="B314" t="n">
-        <v>0.09229539120648336</v>
+        <v>0.1055187403718371</v>
       </c>
     </row>
     <row r="315">
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="B315" t="n">
-        <v>0.1069855156445302</v>
+        <v>0.1237366541990808</v>
       </c>
     </row>
     <row r="316">
@@ -3587,7 +3587,7 @@
         </is>
       </c>
       <c r="B316" t="n">
-        <v>0.02024690937175482</v>
+        <v>0.03841370062733952</v>
       </c>
     </row>
     <row r="317">
@@ -3597,7 +3597,7 @@
         </is>
       </c>
       <c r="B317" t="n">
-        <v>0.0653954066126647</v>
+        <v>0.139632709354782</v>
       </c>
     </row>
     <row r="318">
@@ -3607,7 +3607,7 @@
         </is>
       </c>
       <c r="B318" t="n">
-        <v>0.00513757402470809</v>
+        <v>0.1178381145731987</v>
       </c>
     </row>
     <row r="319">
@@ -3617,7 +3617,7 @@
         </is>
       </c>
       <c r="B319" t="n">
-        <v>0.1050553849640236</v>
+        <v>0.1261613145528952</v>
       </c>
     </row>
     <row r="320">
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="B320" t="n">
-        <v>0.05623415596691304</v>
+        <v>0.1098128339398641</v>
       </c>
     </row>
     <row r="321">
@@ -3637,7 +3637,7 @@
         </is>
       </c>
       <c r="B321" t="n">
-        <v>0.02490124938569762</v>
+        <v>0.0812290545553614</v>
       </c>
     </row>
     <row r="322">
@@ -3647,7 +3647,7 @@
         </is>
       </c>
       <c r="B322" t="n">
-        <v>0.06271590160406719</v>
+        <v>0.0976328371578366</v>
       </c>
     </row>
     <row r="323">
@@ -3657,7 +3657,7 @@
         </is>
       </c>
       <c r="B323" t="n">
-        <v>0.01800516884226066</v>
+        <v>0.05966209897617428</v>
       </c>
     </row>
     <row r="324">
@@ -3667,7 +3667,7 @@
         </is>
       </c>
       <c r="B324" t="n">
-        <v>0.0248888047878698</v>
+        <v>0.1066060267413161</v>
       </c>
     </row>
     <row r="325">
@@ -3677,7 +3677,7 @@
         </is>
       </c>
       <c r="B325" t="n">
-        <v>0.08382173377029541</v>
+        <v>0.1450193373204529</v>
       </c>
     </row>
     <row r="326">
@@ -3687,7 +3687,7 @@
         </is>
       </c>
       <c r="B326" t="n">
-        <v>0.01765462603436291</v>
+        <v>0.1256690461368665</v>
       </c>
     </row>
     <row r="327">
@@ -3697,7 +3697,7 @@
         </is>
       </c>
       <c r="B327" t="n">
-        <v>0.002695262253104601</v>
+        <v>0.1942296203032207</v>
       </c>
     </row>
     <row r="328">
@@ -3707,7 +3707,7 @@
         </is>
       </c>
       <c r="B328" t="n">
-        <v>0</v>
+        <v>0.04466720536605549</v>
       </c>
     </row>
     <row r="329">
@@ -3717,7 +3717,7 @@
         </is>
       </c>
       <c r="B329" t="n">
-        <v>0.2124707816666457</v>
+        <v>0.1623683324652578</v>
       </c>
     </row>
     <row r="330">
@@ -3727,7 +3727,7 @@
         </is>
       </c>
       <c r="B330" t="n">
-        <v>0.01525688063724863</v>
+        <v>0.1012491998379259</v>
       </c>
     </row>
     <row r="331">
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="B331" t="n">
-        <v>0.05634863913722681</v>
+        <v>0.09367208925440532</v>
       </c>
     </row>
     <row r="332">
@@ -3747,7 +3747,7 @@
         </is>
       </c>
       <c r="B332" t="n">
-        <v>0.01008702872139817</v>
+        <v>0.1214035791304324</v>
       </c>
     </row>
     <row r="333">
@@ -3757,7 +3757,7 @@
         </is>
       </c>
       <c r="B333" t="n">
-        <v>0.1328508612498616</v>
+        <v>0.219042556400052</v>
       </c>
     </row>
     <row r="334">
@@ -3767,7 +3767,7 @@
         </is>
       </c>
       <c r="B334" t="n">
-        <v>0.07364403945264811</v>
+        <v>0.09155140702071005</v>
       </c>
     </row>
     <row r="335">
@@ -3777,7 +3777,7 @@
         </is>
       </c>
       <c r="B335" t="n">
-        <v>0.009074936433832457</v>
+        <v>0.08777696139589714</v>
       </c>
     </row>
     <row r="336">
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="B336" t="n">
-        <v>0.1135113547492278</v>
+        <v>0.2180771357209378</v>
       </c>
     </row>
     <row r="337">
@@ -3797,7 +3797,7 @@
         </is>
       </c>
       <c r="B337" t="n">
-        <v>0.01450903023908238</v>
+        <v>0.08587822543910141</v>
       </c>
     </row>
     <row r="338">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="B338" t="n">
-        <v>0.1127715756809027</v>
+        <v>0.1706185256639669</v>
       </c>
     </row>
     <row r="339">
@@ -3817,7 +3817,7 @@
         </is>
       </c>
       <c r="B339" t="n">
-        <v>0.06931176343385839</v>
+        <v>0.08628660218767581</v>
       </c>
     </row>
     <row r="340">
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="B340" t="n">
-        <v>0.03620226527034785</v>
+        <v>0.07538868395506026</v>
       </c>
     </row>
     <row r="341">
@@ -3837,7 +3837,7 @@
         </is>
       </c>
       <c r="B341" t="n">
-        <v>0.07094831250378925</v>
+        <v>0.1204927216360911</v>
       </c>
     </row>
     <row r="342">
@@ -3847,7 +3847,7 @@
         </is>
       </c>
       <c r="B342" t="n">
-        <v>0.05637373168408395</v>
+        <v>0.1533899473514956</v>
       </c>
     </row>
     <row r="343">
@@ -3857,7 +3857,7 @@
         </is>
       </c>
       <c r="B343" t="n">
-        <v>0.08472718979844121</v>
+        <v>0.144665775297138</v>
       </c>
     </row>
     <row r="344">
@@ -3867,7 +3867,7 @@
         </is>
       </c>
       <c r="B344" t="n">
-        <v>0.09464494285908849</v>
+        <v>0.1806168538779697</v>
       </c>
     </row>
     <row r="345">
@@ -3877,7 +3877,7 @@
         </is>
       </c>
       <c r="B345" t="n">
-        <v>0.07117803565951419</v>
+        <v>0.08563847165120203</v>
       </c>
     </row>
     <row r="346">
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="B346" t="n">
-        <v>0.06056331193857192</v>
+        <v>0.128613759671024</v>
       </c>
     </row>
     <row r="347">
@@ -3897,7 +3897,7 @@
         </is>
       </c>
       <c r="B347" t="n">
-        <v>0.040539422311269</v>
+        <v>0.09572488869986151</v>
       </c>
     </row>
     <row r="348">
@@ -3907,7 +3907,7 @@
         </is>
       </c>
       <c r="B348" t="n">
-        <v>0.04498644663176957</v>
+        <v>0.1276253231053479</v>
       </c>
     </row>
     <row r="349">
@@ -3917,7 +3917,7 @@
         </is>
       </c>
       <c r="B349" t="n">
-        <v>0.02520205441032976</v>
+        <v>0.09312729777191386</v>
       </c>
     </row>
     <row r="350">
@@ -3927,7 +3927,7 @@
         </is>
       </c>
       <c r="B350" t="n">
-        <v>0.06040955087562747</v>
+        <v>0.1849163715903324</v>
       </c>
     </row>
     <row r="351">
@@ -3937,7 +3937,7 @@
         </is>
       </c>
       <c r="B351" t="n">
-        <v>0.005290774738310428</v>
+        <v>0.04011419903151503</v>
       </c>
     </row>
     <row r="352">
@@ -3947,7 +3947,7 @@
         </is>
       </c>
       <c r="B352" t="n">
-        <v>0.04412731419419769</v>
+        <v>0.1564682314096137</v>
       </c>
     </row>
     <row r="353">
@@ -3957,7 +3957,7 @@
         </is>
       </c>
       <c r="B353" t="n">
-        <v>0.008868850189196425</v>
+        <v>0.06576730945006939</v>
       </c>
     </row>
     <row r="354">
@@ -3967,7 +3967,7 @@
         </is>
       </c>
       <c r="B354" t="n">
-        <v>0.04150544123262793</v>
+        <v>0.09898175376474984</v>
       </c>
     </row>
     <row r="355">
@@ -3977,7 +3977,7 @@
         </is>
       </c>
       <c r="B355" t="n">
-        <v>0.04102111962119464</v>
+        <v>0.1505203714375678</v>
       </c>
     </row>
     <row r="356">
@@ -3987,7 +3987,7 @@
         </is>
       </c>
       <c r="B356" t="n">
-        <v>0.02997587631389834</v>
+        <v>0.1491149025978295</v>
       </c>
     </row>
     <row r="357">
@@ -3997,7 +3997,7 @@
         </is>
       </c>
       <c r="B357" t="n">
-        <v>0.02035865701100629</v>
+        <v>0.05532874426268883</v>
       </c>
     </row>
     <row r="358">
@@ -4007,7 +4007,7 @@
         </is>
       </c>
       <c r="B358" t="n">
-        <v>0.0639196174299269</v>
+        <v>0.2847225737050394</v>
       </c>
     </row>
     <row r="359">
@@ -4017,7 +4017,7 @@
         </is>
       </c>
       <c r="B359" t="n">
-        <v>0.06254129728913357</v>
+        <v>0.1194356594290636</v>
       </c>
     </row>
     <row r="360">
@@ -4027,7 +4027,7 @@
         </is>
       </c>
       <c r="B360" t="n">
-        <v>0.005879528775967406</v>
+        <v>0.02171078549038289</v>
       </c>
     </row>
     <row r="361">
@@ -4037,7 +4037,7 @@
         </is>
       </c>
       <c r="B361" t="n">
-        <v>0.0735330335812457</v>
+        <v>0.1090632029458612</v>
       </c>
     </row>
     <row r="362">
@@ -4047,7 +4047,7 @@
         </is>
       </c>
       <c r="B362" t="n">
-        <v>0</v>
+        <v>0.06941048114847052</v>
       </c>
     </row>
     <row r="363">
@@ -4057,7 +4057,7 @@
         </is>
       </c>
       <c r="B363" t="n">
-        <v>0.03917487426568857</v>
+        <v>0.1305965160857962</v>
       </c>
     </row>
     <row r="364">
@@ -4067,7 +4067,7 @@
         </is>
       </c>
       <c r="B364" t="n">
-        <v>0.05872119762099575</v>
+        <v>0.1675509070017901</v>
       </c>
     </row>
     <row r="365">
@@ -4077,7 +4077,7 @@
         </is>
       </c>
       <c r="B365" t="n">
-        <v>0.03842026736970446</v>
+        <v>0.194424592953674</v>
       </c>
     </row>
     <row r="366">
@@ -4087,7 +4087,7 @@
         </is>
       </c>
       <c r="B366" t="n">
-        <v>0.0678339147642909</v>
+        <v>0.1044443731795477</v>
       </c>
     </row>
     <row r="367">
@@ -4097,7 +4097,7 @@
         </is>
       </c>
       <c r="B367" t="n">
-        <v>0.03362689509841292</v>
+        <v>0.05335429383674307</v>
       </c>
     </row>
     <row r="368">
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="B368" t="n">
-        <v>0.01881022853314103</v>
+        <v>0.07412821619927826</v>
       </c>
     </row>
     <row r="369">
@@ -4117,7 +4117,7 @@
         </is>
       </c>
       <c r="B369" t="n">
-        <v>0.03686079038893292</v>
+        <v>0.1129495225851784</v>
       </c>
     </row>
     <row r="370">
@@ -4127,7 +4127,7 @@
         </is>
       </c>
       <c r="B370" t="n">
-        <v>0.0325900630058553</v>
+        <v>0.08774646012864243</v>
       </c>
     </row>
     <row r="371">
@@ -4137,7 +4137,7 @@
         </is>
       </c>
       <c r="B371" t="n">
-        <v>0.01468677523370061</v>
+        <v>0.06686838862274598</v>
       </c>
     </row>
     <row r="372">
@@ -4147,7 +4147,7 @@
         </is>
       </c>
       <c r="B372" t="n">
-        <v>0.06850876531993554</v>
+        <v>0.1695189511341354</v>
       </c>
     </row>
     <row r="373">
@@ -4157,7 +4157,7 @@
         </is>
       </c>
       <c r="B373" t="n">
-        <v>0.04178632969557725</v>
+        <v>0.09571174687818651</v>
       </c>
     </row>
     <row r="374">
@@ -4167,7 +4167,7 @@
         </is>
       </c>
       <c r="B374" t="n">
-        <v>0.01980930512724971</v>
+        <v>0.0566349376288678</v>
       </c>
     </row>
     <row r="375">
@@ -4177,7 +4177,7 @@
         </is>
       </c>
       <c r="B375" t="n">
-        <v>0.06615267239801938</v>
+        <v>0.124910209258099</v>
       </c>
     </row>
     <row r="376">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="B376" t="n">
-        <v>0.08572949288837566</v>
+        <v>0.1813661912222831</v>
       </c>
     </row>
     <row r="377">
@@ -4197,7 +4197,7 @@
         </is>
       </c>
       <c r="B377" t="n">
-        <v>0.07726962547445927</v>
+        <v>0.1801084972471296</v>
       </c>
     </row>
     <row r="378">
@@ -4207,7 +4207,7 @@
         </is>
       </c>
       <c r="B378" t="n">
-        <v>0.07848995622673263</v>
+        <v>0.1200628651759666</v>
       </c>
     </row>
     <row r="379">
@@ -4217,7 +4217,7 @@
         </is>
       </c>
       <c r="B379" t="n">
-        <v>0.03283187844152755</v>
+        <v>0.08340111950643368</v>
       </c>
     </row>
     <row r="380">
@@ -4227,7 +4227,7 @@
         </is>
       </c>
       <c r="B380" t="n">
-        <v>0.01630105801451325</v>
+        <v>0.1015176758066783</v>
       </c>
     </row>
     <row r="381">
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="B381" t="n">
-        <v>0.07735993425830344</v>
+        <v>0.1491875483642526</v>
       </c>
     </row>
     <row r="382">
@@ -4247,7 +4247,7 @@
         </is>
       </c>
       <c r="B382" t="n">
-        <v>0.02349541226677775</v>
+        <v>0.145967903064175</v>
       </c>
     </row>
     <row r="383">
@@ -4257,7 +4257,7 @@
         </is>
       </c>
       <c r="B383" t="n">
-        <v>0.08526170027662372</v>
+        <v>0.1612503932951752</v>
       </c>
     </row>
     <row r="384">
@@ -4267,7 +4267,7 @@
         </is>
       </c>
       <c r="B384" t="n">
-        <v>0.04805171826957261</v>
+        <v>0.1619366345933005</v>
       </c>
     </row>
     <row r="385">
@@ -4277,7 +4277,7 @@
         </is>
       </c>
       <c r="B385" t="n">
-        <v>0.01156870758682783</v>
+        <v>0.05853868321407645</v>
       </c>
     </row>
     <row r="386">
@@ -4287,7 +4287,7 @@
         </is>
       </c>
       <c r="B386" t="n">
-        <v>0.08872569844900233</v>
+        <v>0.2010394255012311</v>
       </c>
     </row>
     <row r="387">
@@ -4297,7 +4297,7 @@
         </is>
       </c>
       <c r="B387" t="n">
-        <v>0.00202253709181905</v>
+        <v>0.03960647541161087</v>
       </c>
     </row>
     <row r="388">
@@ -4307,7 +4307,7 @@
         </is>
       </c>
       <c r="B388" t="n">
-        <v>0.02973838202537243</v>
+        <v>0.09092938784184544</v>
       </c>
     </row>
     <row r="389">
@@ -4317,7 +4317,7 @@
         </is>
       </c>
       <c r="B389" t="n">
-        <v>0.05672129160072317</v>
+        <v>0.07224362601965921</v>
       </c>
     </row>
     <row r="390">
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="B390" t="n">
-        <v>0.06065942869612908</v>
+        <v>0.2194402359591982</v>
       </c>
     </row>
     <row r="391">
@@ -4337,7 +4337,7 @@
         </is>
       </c>
       <c r="B391" t="n">
-        <v>0</v>
+        <v>0.0709445151232171</v>
       </c>
     </row>
     <row r="392">
@@ -4347,7 +4347,7 @@
         </is>
       </c>
       <c r="B392" t="n">
-        <v>0.06050474033473392</v>
+        <v>0.2848249952887397</v>
       </c>
     </row>
     <row r="393">
@@ -4357,7 +4357,7 @@
         </is>
       </c>
       <c r="B393" t="n">
-        <v>0.1241970466354477</v>
+        <v>0.1506540527529256</v>
       </c>
     </row>
     <row r="394">
@@ -4367,7 +4367,7 @@
         </is>
       </c>
       <c r="B394" t="n">
-        <v>0.03442121332909014</v>
+        <v>0.08322357809772302</v>
       </c>
     </row>
     <row r="395">
@@ -4377,7 +4377,7 @@
         </is>
       </c>
       <c r="B395" t="n">
-        <v>0.01249435837824776</v>
+        <v>0.05165641003272391</v>
       </c>
     </row>
     <row r="396">
@@ -4387,7 +4387,7 @@
         </is>
       </c>
       <c r="B396" t="n">
-        <v>0.04033653770714933</v>
+        <v>0.1196012225982559</v>
       </c>
     </row>
     <row r="397">
@@ -4397,7 +4397,7 @@
         </is>
       </c>
       <c r="B397" t="n">
-        <v>0.05707919247232507</v>
+        <v>0.1406620785610237</v>
       </c>
     </row>
     <row r="398">
@@ -4407,7 +4407,7 @@
         </is>
       </c>
       <c r="B398" t="n">
-        <v>0.07198050965878032</v>
+        <v>0.1660172314847822</v>
       </c>
     </row>
     <row r="399">
@@ -4417,7 +4417,7 @@
         </is>
       </c>
       <c r="B399" t="n">
-        <v>0.04622544518622129</v>
+        <v>0.1439468833137954</v>
       </c>
     </row>
     <row r="400">
@@ -4427,7 +4427,7 @@
         </is>
       </c>
       <c r="B400" t="n">
-        <v>0.1455009395136745</v>
+        <v>0.1185661986371749</v>
       </c>
     </row>
     <row r="401">
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="B401" t="n">
-        <v>0.03730794110433089</v>
+        <v>0.1043748088182754</v>
       </c>
     </row>
     <row r="402">
@@ -4447,7 +4447,7 @@
         </is>
       </c>
       <c r="B402" t="n">
-        <v>0.004137402676073904</v>
+        <v>0.1470246127169623</v>
       </c>
     </row>
     <row r="403">
@@ -4457,7 +4457,7 @@
         </is>
       </c>
       <c r="B403" t="n">
-        <v>0.0567110412144828</v>
+        <v>0.1031054849658259</v>
       </c>
     </row>
     <row r="404">
@@ -4467,7 +4467,7 @@
         </is>
       </c>
       <c r="B404" t="n">
-        <v>0.04392991611130533</v>
+        <v>0.1046144845338468</v>
       </c>
     </row>
     <row r="405">
@@ -4477,7 +4477,7 @@
         </is>
       </c>
       <c r="B405" t="n">
-        <v>0</v>
+        <v>0.05395052336903654</v>
       </c>
     </row>
     <row r="406">
@@ -4487,7 +4487,7 @@
         </is>
       </c>
       <c r="B406" t="n">
-        <v>0.1007106339717374</v>
+        <v>0.1745646484418573</v>
       </c>
     </row>
     <row r="407">
@@ -4497,7 +4497,7 @@
         </is>
       </c>
       <c r="B407" t="n">
-        <v>0.04980754840763146</v>
+        <v>0.1330089358764181</v>
       </c>
     </row>
     <row r="408">
@@ -4507,7 +4507,7 @@
         </is>
       </c>
       <c r="B408" t="n">
-        <v>0.03091320480509759</v>
+        <v>0.06286284325335019</v>
       </c>
     </row>
     <row r="409">
@@ -4517,7 +4517,7 @@
         </is>
       </c>
       <c r="B409" t="n">
-        <v>0.170542163116391</v>
+        <v>0.2222321859640402</v>
       </c>
     </row>
     <row r="410">
@@ -4527,7 +4527,7 @@
         </is>
       </c>
       <c r="B410" t="n">
-        <v>0.03586231350699736</v>
+        <v>0.1954826726553747</v>
       </c>
     </row>
     <row r="411">
@@ -4537,7 +4537,7 @@
         </is>
       </c>
       <c r="B411" t="n">
-        <v>0.03190853524514001</v>
+        <v>0.08735703153006166</v>
       </c>
     </row>
     <row r="412">
@@ -4547,7 +4547,7 @@
         </is>
       </c>
       <c r="B412" t="n">
-        <v>0.04221122876951438</v>
+        <v>0.08705325132445892</v>
       </c>
     </row>
     <row r="413">
@@ -4557,7 +4557,7 @@
         </is>
       </c>
       <c r="B413" t="n">
-        <v>0.08085374146986558</v>
+        <v>0.2123599931771954</v>
       </c>
     </row>
     <row r="414">
@@ -4567,7 +4567,7 @@
         </is>
       </c>
       <c r="B414" t="n">
-        <v>0.0745374449339207</v>
+        <v>0.1118069671330642</v>
       </c>
     </row>
     <row r="415">
@@ -4577,7 +4577,7 @@
         </is>
       </c>
       <c r="B415" t="n">
-        <v>0.0749862026991225</v>
+        <v>0.2042697543062919</v>
       </c>
     </row>
     <row r="416">
@@ -4587,7 +4587,7 @@
         </is>
       </c>
       <c r="B416" t="n">
-        <v>0.170816336506787</v>
+        <v>0.2954976898346023</v>
       </c>
     </row>
     <row r="417">
@@ -4597,7 +4597,7 @@
         </is>
       </c>
       <c r="B417" t="n">
-        <v>0.06645825457198477</v>
+        <v>0.1661043427063024</v>
       </c>
     </row>
     <row r="418">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="B418" t="n">
-        <v>0.1401376467401358</v>
+        <v>0.1825933295608263</v>
       </c>
     </row>
     <row r="419">
@@ -4617,7 +4617,7 @@
         </is>
       </c>
       <c r="B419" t="n">
-        <v>0.1208993755062686</v>
+        <v>0.2162268792390524</v>
       </c>
     </row>
     <row r="420">
@@ -4627,7 +4627,7 @@
         </is>
       </c>
       <c r="B420" t="n">
-        <v>0.05790898512901928</v>
+        <v>0.08117305251975197</v>
       </c>
     </row>
     <row r="421">
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="B421" t="n">
-        <v>0.03914601787808899</v>
+        <v>0.0460611876665008</v>
       </c>
     </row>
     <row r="422">
@@ -4647,7 +4647,7 @@
         </is>
       </c>
       <c r="B422" t="n">
-        <v>0.1064355821034391</v>
+        <v>0.1947938143724725</v>
       </c>
     </row>
     <row r="423">
@@ -4657,7 +4657,7 @@
         </is>
       </c>
       <c r="B423" t="n">
-        <v>0.007076932147342962</v>
+        <v>0.07029628672310452</v>
       </c>
     </row>
     <row r="424">
@@ -4667,7 +4667,7 @@
         </is>
       </c>
       <c r="B424" t="n">
-        <v>0.01279053605784932</v>
+        <v>0.05499550990958692</v>
       </c>
     </row>
     <row r="425">
@@ -4677,7 +4677,7 @@
         </is>
       </c>
       <c r="B425" t="n">
-        <v>0.2271200985034241</v>
+        <v>0.2025052820490396</v>
       </c>
     </row>
     <row r="426">
@@ -4687,7 +4687,7 @@
         </is>
       </c>
       <c r="B426" t="n">
-        <v>0.08310625481653436</v>
+        <v>0.08915618200352125</v>
       </c>
     </row>
     <row r="427">
@@ -4697,7 +4697,7 @@
         </is>
       </c>
       <c r="B427" t="n">
-        <v>0.0411543741013236</v>
+        <v>0.1288802040945017</v>
       </c>
     </row>
     <row r="428">
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="B428" t="n">
-        <v>0.04325627946376798</v>
+        <v>0.1554985360237752</v>
       </c>
     </row>
     <row r="429">
@@ -4717,7 +4717,7 @@
         </is>
       </c>
       <c r="B429" t="n">
-        <v>0.03826800756075917</v>
+        <v>0.1172021967931354</v>
       </c>
     </row>
     <row r="430">
@@ -4727,7 +4727,7 @@
         </is>
       </c>
       <c r="B430" t="n">
-        <v>0.03243044134774069</v>
+        <v>0.1014318304856975</v>
       </c>
     </row>
     <row r="431">
@@ -4737,7 +4737,7 @@
         </is>
       </c>
       <c r="B431" t="n">
-        <v>0.1068664959242878</v>
+        <v>0.1614701005283943</v>
       </c>
     </row>
     <row r="432">
@@ -4747,7 +4747,7 @@
         </is>
       </c>
       <c r="B432" t="n">
-        <v>0.06610968980699627</v>
+        <v>0.1425182354184797</v>
       </c>
     </row>
     <row r="433">
@@ -4757,7 +4757,7 @@
         </is>
       </c>
       <c r="B433" t="n">
-        <v>0.01815520024188962</v>
+        <v>0.1101797098986317</v>
       </c>
     </row>
     <row r="434">
@@ -4767,7 +4767,7 @@
         </is>
       </c>
       <c r="B434" t="n">
-        <v>0.03569267636333387</v>
+        <v>0.1283974395929715</v>
       </c>
     </row>
     <row r="435">
@@ -4777,7 +4777,7 @@
         </is>
       </c>
       <c r="B435" t="n">
-        <v>0.02077601725264858</v>
+        <v>0.1189497079883483</v>
       </c>
     </row>
     <row r="436">
@@ -4787,7 +4787,7 @@
         </is>
       </c>
       <c r="B436" t="n">
-        <v>0.05023407113440044</v>
+        <v>0.2021647334093536</v>
       </c>
     </row>
     <row r="437">
@@ -4797,7 +4797,7 @@
         </is>
       </c>
       <c r="B437" t="n">
-        <v>0.04840980553372708</v>
+        <v>0.1552382243413986</v>
       </c>
     </row>
     <row r="438">
@@ -4807,7 +4807,7 @@
         </is>
       </c>
       <c r="B438" t="n">
-        <v>0.01651538769338957</v>
+        <v>0.1019388305275096</v>
       </c>
     </row>
     <row r="439">
@@ -4817,7 +4817,7 @@
         </is>
       </c>
       <c r="B439" t="n">
-        <v>0.06430355319403633</v>
+        <v>0.1654645624102592</v>
       </c>
     </row>
     <row r="440">
@@ -4827,7 +4827,7 @@
         </is>
       </c>
       <c r="B440" t="n">
-        <v>0.09072812455627602</v>
+        <v>0.1215731547381136</v>
       </c>
     </row>
     <row r="441">
@@ -4837,7 +4837,7 @@
         </is>
       </c>
       <c r="B441" t="n">
-        <v>0.1021367683433411</v>
+        <v>0.1734550157625831</v>
       </c>
     </row>
     <row r="442">
@@ -4847,7 +4847,7 @@
         </is>
       </c>
       <c r="B442" t="n">
-        <v>0.07417126704692209</v>
+        <v>0.06573061694731686</v>
       </c>
     </row>
     <row r="443">
@@ -4857,7 +4857,7 @@
         </is>
       </c>
       <c r="B443" t="n">
-        <v>0.09649609211260024</v>
+        <v>0.1793791219364756</v>
       </c>
     </row>
     <row r="444">
@@ -4867,7 +4867,7 @@
         </is>
       </c>
       <c r="B444" t="n">
-        <v>0.06681914446810289</v>
+        <v>0.221593918928298</v>
       </c>
     </row>
     <row r="445">
@@ -4877,7 +4877,7 @@
         </is>
       </c>
       <c r="B445" t="n">
-        <v>0.08881926626663972</v>
+        <v>0.1614568125418986</v>
       </c>
     </row>
     <row r="446">
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="B446" t="n">
-        <v>0.03148275201886713</v>
+        <v>0.1339319871501546</v>
       </c>
     </row>
     <row r="447">
@@ -4897,7 +4897,7 @@
         </is>
       </c>
       <c r="B447" t="n">
-        <v>0.1295668833727625</v>
+        <v>0.1301800310047478</v>
       </c>
     </row>
     <row r="448">
@@ -4907,7 +4907,7 @@
         </is>
       </c>
       <c r="B448" t="n">
-        <v>0.02009751236002226</v>
+        <v>0.1718136945480628</v>
       </c>
     </row>
     <row r="449">
@@ -4917,7 +4917,7 @@
         </is>
       </c>
       <c r="B449" t="n">
-        <v>0.0231454672107667</v>
+        <v>0.08159806252042286</v>
       </c>
     </row>
     <row r="450">
@@ -4927,7 +4927,7 @@
         </is>
       </c>
       <c r="B450" t="n">
-        <v>0.00802076655228327</v>
+        <v>0.06244622372585346</v>
       </c>
     </row>
     <row r="451">
@@ -4937,7 +4937,7 @@
         </is>
       </c>
       <c r="B451" t="n">
-        <v>0</v>
+        <v>0.2146741416696738</v>
       </c>
     </row>
     <row r="452">
@@ -4947,7 +4947,7 @@
         </is>
       </c>
       <c r="B452" t="n">
-        <v>0.03117593725247008</v>
+        <v>0.1550051538629873</v>
       </c>
     </row>
     <row r="453">
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="B453" t="n">
-        <v>0.02498827424486637</v>
+        <v>0.03870473982868012</v>
       </c>
     </row>
     <row r="454">
@@ -4967,7 +4967,7 @@
         </is>
       </c>
       <c r="B454" t="n">
-        <v>0.03721358890545495</v>
+        <v>0.112983036976536</v>
       </c>
     </row>
     <row r="455">
@@ -4977,7 +4977,7 @@
         </is>
       </c>
       <c r="B455" t="n">
-        <v>0.01167591879100291</v>
+        <v>0.1022903886187686</v>
       </c>
     </row>
     <row r="456">
@@ -4987,7 +4987,7 @@
         </is>
       </c>
       <c r="B456" t="n">
-        <v>0.05046711237522354</v>
+        <v>0.1222912072164841</v>
       </c>
     </row>
     <row r="457">
@@ -4997,7 +4997,7 @@
         </is>
       </c>
       <c r="B457" t="n">
-        <v>0.06645756234588666</v>
+        <v>0.1625904944198339</v>
       </c>
     </row>
     <row r="458">
@@ -5007,7 +5007,7 @@
         </is>
       </c>
       <c r="B458" t="n">
-        <v>0.05483843587630544</v>
+        <v>0.1061063699638992</v>
       </c>
     </row>
     <row r="459">
@@ -5017,7 +5017,7 @@
         </is>
       </c>
       <c r="B459" t="n">
-        <v>0.1102505373600981</v>
+        <v>0.188660196942241</v>
       </c>
     </row>
     <row r="460">
@@ -5027,7 +5027,7 @@
         </is>
       </c>
       <c r="B460" t="n">
-        <v>0.05427396233642125</v>
+        <v>0.07989245231261556</v>
       </c>
     </row>
     <row r="461">
@@ -5037,7 +5037,7 @@
         </is>
       </c>
       <c r="B461" t="n">
-        <v>0.1004835743790337</v>
+        <v>0.1770679894501551</v>
       </c>
     </row>
     <row r="462">
@@ -5047,7 +5047,7 @@
         </is>
       </c>
       <c r="B462" t="n">
-        <v>0.04285373954713621</v>
+        <v>0.02695599155598598</v>
       </c>
     </row>
     <row r="463">
@@ -5057,7 +5057,7 @@
         </is>
       </c>
       <c r="B463" t="n">
-        <v>0.02422046720585325</v>
+        <v>0.1290037330638924</v>
       </c>
     </row>
     <row r="464">
@@ -5067,7 +5067,7 @@
         </is>
       </c>
       <c r="B464" t="n">
-        <v>0.0379445910890053</v>
+        <v>0.1696754768901337</v>
       </c>
     </row>
     <row r="465">
@@ -5077,7 +5077,7 @@
         </is>
       </c>
       <c r="B465" t="n">
-        <v>0.1202298702688091</v>
+        <v>0.189104421078074</v>
       </c>
     </row>
     <row r="466">
@@ -5087,7 +5087,7 @@
         </is>
       </c>
       <c r="B466" t="n">
-        <v>0</v>
+        <v>0.02548914182456321</v>
       </c>
     </row>
     <row r="467">
@@ -5097,7 +5097,7 @@
         </is>
       </c>
       <c r="B467" t="n">
-        <v>0.0227543418277264</v>
+        <v>0.06950443600331843</v>
       </c>
     </row>
     <row r="468">
@@ -5107,7 +5107,7 @@
         </is>
       </c>
       <c r="B468" t="n">
-        <v>0.03987748029888281</v>
+        <v>0.09458279392659147</v>
       </c>
     </row>
     <row r="469">
@@ -5117,7 +5117,7 @@
         </is>
       </c>
       <c r="B469" t="n">
-        <v>0.03045787424384923</v>
+        <v>0.1646581659350195</v>
       </c>
     </row>
     <row r="470">
@@ -5127,7 +5127,7 @@
         </is>
       </c>
       <c r="B470" t="n">
-        <v>0.1049263389077578</v>
+        <v>0.1710844523294623</v>
       </c>
     </row>
     <row r="471">
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="B471" t="n">
-        <v>0.04231565509534749</v>
+        <v>0.1151293478344385</v>
       </c>
     </row>
     <row r="472">
@@ -5147,7 +5147,7 @@
         </is>
       </c>
       <c r="B472" t="n">
-        <v>0.0140055669097524</v>
+        <v>0.1219386347167586</v>
       </c>
     </row>
     <row r="473">
@@ -5157,7 +5157,7 @@
         </is>
       </c>
       <c r="B473" t="n">
-        <v>0.07063793721480109</v>
+        <v>0.09367318193516416</v>
       </c>
     </row>
     <row r="474">
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="B474" t="n">
-        <v>0.05644119597160523</v>
+        <v>0.1738455152784515</v>
       </c>
     </row>
     <row r="475">
@@ -5177,7 +5177,7 @@
         </is>
       </c>
       <c r="B475" t="n">
-        <v>0.04241822091016732</v>
+        <v>0.06573736797493934</v>
       </c>
     </row>
     <row r="476">
@@ -5187,7 +5187,7 @@
         </is>
       </c>
       <c r="B476" t="n">
-        <v>0.0555092076622826</v>
+        <v>0.2313331858803513</v>
       </c>
     </row>
     <row r="477">
@@ -5197,7 +5197,7 @@
         </is>
       </c>
       <c r="B477" t="n">
-        <v>0.01776935342935605</v>
+        <v>0.04605547205525126</v>
       </c>
     </row>
     <row r="478">
@@ -5207,7 +5207,7 @@
         </is>
       </c>
       <c r="B478" t="n">
-        <v>0.05454941414851559</v>
+        <v>0.06700550164084262</v>
       </c>
     </row>
     <row r="479">
@@ -5217,7 +5217,7 @@
         </is>
       </c>
       <c r="B479" t="n">
-        <v>0.04783854796597101</v>
+        <v>0.1375940996085052</v>
       </c>
     </row>
     <row r="480">
@@ -5227,7 +5227,7 @@
         </is>
       </c>
       <c r="B480" t="n">
-        <v>0</v>
+        <v>0.02121011208035121</v>
       </c>
     </row>
     <row r="481">
@@ -5237,7 +5237,7 @@
         </is>
       </c>
       <c r="B481" t="n">
-        <v>0.03751778264448626</v>
+        <v>0.1007677877093383</v>
       </c>
     </row>
     <row r="482">
@@ -5247,7 +5247,7 @@
         </is>
       </c>
       <c r="B482" t="n">
-        <v>0.04176975245046916</v>
+        <v>0.174496123015982</v>
       </c>
     </row>
     <row r="483">
@@ -5257,7 +5257,7 @@
         </is>
       </c>
       <c r="B483" t="n">
-        <v>0.01908344993799694</v>
+        <v>0.07101936376588355</v>
       </c>
     </row>
     <row r="484">
@@ -5267,7 +5267,7 @@
         </is>
       </c>
       <c r="B484" t="n">
-        <v>0.0237186579844877</v>
+        <v>0.08337578718566387</v>
       </c>
     </row>
     <row r="485">
@@ -5277,7 +5277,7 @@
         </is>
       </c>
       <c r="B485" t="n">
-        <v>0.0448751499103594</v>
+        <v>0.1618285548308269</v>
       </c>
     </row>
   </sheetData>

</xml_diff>